<commit_message>
Lock Stuffcool run: approved data, validated images, build checks, and 7-page PDF output
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL1"/>
+  <dimension ref="A1:AM11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,6 +605,1235 @@
       <c r="AL1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Image_Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PB-SC-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Aura</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>2099</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/aura-10000mah-15w-magnetic-wireless-powerbank-with-gold-finish</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Stuffcool Aura 10000mAh Power Bank</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>15W Magnetic Wireless &amp; 20W PD Fast Charging Powerbank</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>3999</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>10,000 mAh</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>15W Wireless / 20W PD Type-C</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1 x Type-C (Input/Output)</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>181g ± 10g</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 1 Year)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>10,000mAh capacity with a stylish gold finish</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Up to 15W magnetic wireless charging for MagSafe</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>20W PD fast charging: 0 to 50% iPhone charge in 30 mins</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>BIS-certified, pocket-friendly and made in India</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>specs: brand-site (stuffcool.com) (https://www.stuffcool.com/products/aura-10000mah-15w-magnetic-wireless-powerbank-with-gold-finish) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>http://www.stuffcool.com/cdn/shop/files/AuraGold.jpg?v=1763803479&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>brand-site</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PB-SC-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click 10</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1699</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/click-10000mah-15w-slim-magnetic-wireless-powerbank-with-natural-titanium-finish-for-iphone</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Stuffcool Click 10 Powerbank</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>10000mAh 15W Slim Magnetic Wireless Powerbank with 20W PD Charging</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>2999</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>10,000 mAh</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>15W Wireless / 20W PD Wired</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1 x Type-C, 1 x USB-A</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>186g ± 10g</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>6 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>15W magnetic wireless charging for iPhone 12 and above.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>20W PD fast charging boosts iPhone to 50% in 30 mins.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Features Type-C and USB-A ports to charge multi-devices.</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>BIS certified with built-in safety, proudly Made in India.</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>specs: brand-site (stuffcool.com) (https://www.stuffcool.com/products/click-10000mah-15w-slim-magnetic-wireless-powerbank-with-natural-titanium-finish-for-iphone) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>http://www.stuffcool.com/cdn/shop/files/Click_10B.jpg?v=1767854721&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>brand-site</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PB-SC-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Giga 20000 mAH</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/giga-65w-20000-mah-qcpd-powerbank-with-type-c-cable</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>2899</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Manual entry — official page delisted</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Stuffcool Giga 20000 mAh Powerbank</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>High-capacity powerbank from Stuffcool for all your devices</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>5999</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>20,000 mAh</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>High 20,000 mAh battery capacity to charge your devices.</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Reliable accessory from leading Indian brand Stuffcool.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Designed for seamless power backup on the go.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Compatible with smartphones and electronic devices.</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>specs: manual-product-url (https://www.stuffcool.com/products/giga-65w-20000-mah-qcpd-powerbank-with-type-c-cable) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/512-Gzw0y5L._SL1500_.jpg</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Stuffcool Giga 20000mAh Powerbank</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>20000mAh 65W laptop powerbank with built-in Type-C cable</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>20,000 mAh</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>65W Power Delivery (built-in cable), 18W USB-A</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Built-in Type-C Cable, 1 x USB-A</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>380g (10.8 x 6.8 x 3.25 cm)</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 1 Year)</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Built-in 65W Type-C cable charges MacBooks and laptops.</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>20,000mAh in one of the smallest bodies in its class.</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Supports 45W Samsung Super Fast Charging 2.0.</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>45W fast input recharges the powerbank quickly.</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>amazon.in/dp/B0DMDZF5SV</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PB-SC-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Lucid</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/lucid-15w-magnetic-wireless-powerbank-5000mah-battery-capacity-for-iphone-16-15-14-13-and-12</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1699</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Manual entry — official page delisted</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Stuffcool Lucid Charging Accessory</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>High-quality charging solutions from India's trusted brand</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Homegrown Indian charging accessories brand</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Reliable &amp; durable accessories for devices</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Nationwide free shipping on orders over Rs 399</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Seamless customer support available via WhatsApp</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>specs: manual-product-url (https://www.stuffcool.com/products/lucid-15w-magnetic-wireless-powerbank-5000mah-battery-capacity-for-iphone-16-15-14-13-and-12) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Stuffcool Lucid 5000mAh Powerbank</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>5000mAh 15W magnetic wireless powerbank, ultra-compact</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>5,000 mAh / 19.25Wh</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>15W Wireless, 20W Type-C PD</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>1 x Type-C (Input/Output)</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>105g ± 10g (7.7 x 6.6 x 2.05 cm)</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 1 Year)</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Smallest 5000mAh magnetic wireless powerbank.</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>15W magnetic wireless charging for iPhone 12 and above.</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>20W PD wired charging delivers 50% in 30 minutes.</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>Breathable LED indicator shows power level at a glance.</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>local-disk</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PB-SC-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Major 10000 mAH</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/major-10000mah-20w-pd-powerbank</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>849</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Manual entry — official page delisted</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Stuffcool Major 10000mAh Powerbank</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Reliable and durable 10000mAh charging accessory for modern smartphones</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>4990</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>10,000 mAh</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>10,000mAh capacity for reliable portable power.</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Homegrown Indian brand offering high-quality products.</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Reliable and durable accessory for daily charging.</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Nationwide free shipping on orders above Rs. 399.</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>specs: manual-product-url (https://www.stuffcool.com/products/major-10000mah-20w-pd-powerbank) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Stuffcool Major 10000mAh Powerbank</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>10000mAh 20W PD powerbank with four charging ports</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>10,000 mAh</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>20W Type-C PD, 22.5W QC3.0 USB-A</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>1 x Type-C (Input/Output), 1 x Micro-USB (Input), 2 x USB-A</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>230g (14 x 6.8 x 1.74 cm)</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 1 Year)</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>10,000mAh slim powerbank, proudly Made in India.</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>20W Type-C PD charges iPhone to 50% in 30 mins.</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>22.5W QC3.0 USB-A for Android fast charging.</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Four ports charge multiple devices at once.</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>local-disk</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PB-SC-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Roam Plus</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/roam-20000mah-mini-powerbank-with-20w-type-c-output</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1499</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/roam-20000mah-mini-powerbank-with-20w-type-c-output</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Stuffcool Roam Plus 20000mAh Powerbank</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Compact 20,000mAh mini powerbank with 20W PD fast charging</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>3499</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>20,000 mAh</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>22.5W Max Fast Charging</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1 x Type-C (PD), 1 x USB-A</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>322g ± 10g</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 1 Year)</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>20,000mAh capacity in an ultra-compact travel design</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>20W Type-C PD charges iPhone to 50% in 30 mins</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>22.5W USB-A port for Android universal fast charge</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>BIS-certified &amp; Made in India for ultimate safety</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>specs: manual-product-url (https://www.stuffcool.com/products/roam-20000mah-mini-powerbank-with-20w-type-c-output) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>http://www.stuffcool.com/cdn/shop/files/Roam_-TN.jpg?v=1747459169&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>brand-site</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PB-SC-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Odin</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>3199</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/odin-10-000mah-qi2-magsafe-powerbank-with-built-in-type-c-cable</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Stuffcool Odin 10000mAh Qi2 Powerbank</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>15W Qi2 MagSafe Wireless Charging with Built-In 35W Type-C Cable</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>4499</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>10,000 mAh</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>35W PD Wired / 15W Wireless</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Built-in Type-C Cable, Type-C Port</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>230g ± 10g</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 12 Months)</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>15W Qi2 MagSafe fast wireless charging for iPhones.</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>35W PD wired charging powers devices to 50% in 30 mins.</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Integrated 35W Type-C cable for complete convenience.</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Includes a built-in phone stand and digital display.</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>specs: brand-site (stuffcool.com) (https://www.stuffcool.com/products/odin-10-000mah-qi2-magsafe-powerbank-with-built-in-type-c-cable) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>http://www.stuffcool.com/cdn/shop/files/Odin.jpg?v=1754635403&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>brand-site</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PB-SC-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1#</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/1-22-5w-10000mah-powerbank-with-20w-pd-type-c-fast-charging</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>949</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/1-22-5w-10000mah-powerbank-with-20w-pd-type-c-fast-charging</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Stuffcool 1# 22.5W 10000mAh Powerbank</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Everyday 22.5W fast charging companion with 20W Type-C PD</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>1899</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>10000mAh/37Wh</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>22.5W (USB-A), 20W PD (Type-C)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1 x Type-C (Input/Output), 1 x USB-A</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>228gm</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Charges compatible iPhones up to 50% in 30 minutes.</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Delivers 22.5W fast charging via USB-A output.</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Supports PD, AFC, FCP, and SCP charging protocols.</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>BIS Approved and Proudly Made in India.</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>specs: manual-product-url (https://www.stuffcool.com/products/1-22-5w-10000mah-powerbank-with-20w-pd-type-c-fast-charging) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>http://www.stuffcool.com/cdn/shop/files/1_White_jpg.jpg?v=1784099782&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 1 Year)</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>brand-site</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PB-SC-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Click 20</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/click-20000mah-15w-magnetic-wireless-powerbank-with-natural-titanium-finish-for-iphone</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2375</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Manual entry — official page delisted</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Stuffcool Click 20</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Reliable &amp; durable charging accessory by Stuffcool</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Reliable and durable brand quality from Stuffcool.</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Designed for today's modern smartphones.</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>High-quality accessories from a leading Indian brand.</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Top quality products built for seamless everyday use.</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>specs: manual-product-url (https://www.stuffcool.com/products/click-20000mah-15w-magnetic-wireless-powerbank-with-natural-titanium-finish-for-iphone) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/51Lo48bbYSL._SL1500_.jpg</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Stuffcool Click 20 Powerbank</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>20000mAh 15W magnetic wireless powerbank with digital display</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>20,000 mAh / 77Wh</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>15W Wireless, 20W Type-C PD with PPS, 18W USB-A</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>1 x Type-C (Input/Output), 1 x USB-A</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>326g ± 10g (11.0 x 6.9 x 2.85 cm)</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 1 Year)</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>India's first 20,000mAh magnetic wireless powerbank.</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>15W magnetic wireless charging for iPhone 12 and above.</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>20W PD wired charging delivers 50% in 30 minutes.</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>Digital display shows exact battery percentage.</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>amazon.in/dp/B0DFZ1KDPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PB-SC-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Stuffcool</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Omni pro</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>3799</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/omni-pro-qi2-2-certified-25w-magsafe-powerbank-with-apple-watch-charger</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Stuffcool Omni Pro 25W Powerbank</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Qi2.2 MagSafe powerbank with built-in Apple Watch charger</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>5999</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>10,000 mAh</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>25W Wireless / 35W USB-C PD</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1 x Type-C (Input/Output)</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>214g ± 10g</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>25W Qi2.2 wireless fast charging for iPhone</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Slide-out built-in Apple Watch charging module</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>35W USB-C PD output supports fast charging</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>10,000mAh capacity with display and kickstand</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>specs: brand-site (stuffcool.com) (https://www.stuffcool.com/products/omni-pro-qi2-2-certified-25w-magsafe-powerbank-with-apple-watch-charger) | mrp: input-sheet</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>http://www.stuffcool.com/cdn/shop/files/Omni_Pro_jpg.jpg?v=1784550011&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>6 Months (Extendable to 1 Year)</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>brand-site</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Larger cards, MRP collection and display, numbering fix, Display_Name column
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CatalogueData" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatalogueData" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM11"/>
+  <dimension ref="A1:BQ11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -612,6 +612,156 @@
           <t>Image_Source</t>
         </is>
       </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>Display_Name</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>MRP_Display</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Source_Title</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Tier_Title</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Source_Subtitle</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>Tier_Subtitle</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>Source_MRP_Scraped</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>Tier_MRP_Scraped</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>Source_Spec_Capacity</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>Tier_Spec_Capacity</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>Source_Spec_Output</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>Tier_Spec_Output</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>Source_Spec_Ports</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>Tier_Spec_Ports</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>Source_Spec_Weight</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>Tier_Spec_Weight</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>Source_Spec_Warranty</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>Tier_Spec_Warranty</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>Source_Bullet_1</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>Tier_Bullet_1</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>Source_Bullet_2</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>Tier_Bullet_2</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>Source_Bullet_3</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>Tier_Bullet_3</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>Source_Bullet_4</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>Tier_Bullet_4</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>Image_Tier</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>Attempts</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>Fix_Log</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>LLM_Provider</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -629,6 +779,9 @@
           <t>Aura</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>2099</v>
       </c>
@@ -710,6 +863,20 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -720,6 +887,42 @@
           <t>brand-site</t>
         </is>
       </c>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/aura-10000mah-15w-magnetic-wireless-powerbank-with-gold-finish</t>
+        </is>
+      </c>
+      <c r="AU2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -737,6 +940,9 @@
           <t>Click 10</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>1699</v>
       </c>
@@ -818,6 +1024,20 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
       <c r="AL3" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -828,6 +1048,42 @@
           <t>brand-site</t>
         </is>
       </c>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/click-10000mah-15w-slim-magnetic-wireless-powerbank-with-natural-titanium-finish-for-iphone</t>
+        </is>
+      </c>
+      <c r="AU3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
+      <c r="BI3" t="inlineStr"/>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -850,6 +1106,8 @@
           <t>https://www.stuffcool.com/products/giga-65w-20000-mah-qcpd-powerbank-with-type-c-cable</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>2899</v>
       </c>
@@ -869,13 +1127,17 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>5999</v>
+        <v>4999</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>20,000 mAh</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>High 20,000 mAh battery capacity to charge your devices.</t>
@@ -921,6 +1183,7 @@
           <t>20000mAh 65W laptop powerbank with built-in Type-C cable</t>
         </is>
       </c>
+      <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr">
         <is>
           <t>20,000 mAh</t>
@@ -966,6 +1229,8 @@
           <t>45W fast input recharges the powerbank quickly.</t>
         </is>
       </c>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -976,6 +1241,46 @@
           <t>amazon.in/dp/B0DMDZF5SV</t>
         </is>
       </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Giga</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>https://www.reliancedigital.in/product/stuffcool-giga-20000-mah-power-bank-with-type-c-cable-black-m84gzd-8975788</t>
+        </is>
+      </c>
+      <c r="AU4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -998,6 +1303,8 @@
           <t>https://www.stuffcool.com/products/lucid-15w-magnetic-wireless-powerbank-5000mah-battery-capacity-for-iphone-16-15-14-13-and-12</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>1699</v>
       </c>
@@ -1016,6 +1323,14 @@
           <t>High-quality charging solutions from India's trusted brand</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>2499</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
           <t>Homegrown Indian charging accessories brand</t>
@@ -1041,6 +1356,7 @@
           <t>specs: manual-product-url (https://www.stuffcool.com/products/lucid-15w-magnetic-wireless-powerbank-5000mah-battery-capacity-for-iphone-16-15-14-13-and-12) | mrp: input-sheet</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
           <t>ok</t>
@@ -1056,6 +1372,7 @@
           <t>5000mAh 15W magnetic wireless powerbank, ultra-compact</t>
         </is>
       </c>
+      <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr">
         <is>
           <t>5,000 mAh / 19.25Wh</t>
@@ -1101,6 +1418,8 @@
           <t>Breathable LED indicator shows power level at a glance.</t>
         </is>
       </c>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1111,6 +1430,42 @@
           <t>local-disk</t>
         </is>
       </c>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>https://www.reliancedigital.in/product/stuffcool-lucid-5000-mah-magsafe-power-bank-white-m7lij2-8945425</t>
+        </is>
+      </c>
+      <c r="AU5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1133,6 +1488,8 @@
           <t>https://www.stuffcool.com/products/major-10000mah-20w-pd-powerbank</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>849</v>
       </c>
@@ -1151,14 +1508,16 @@
           <t>Reliable and durable 10000mAh charging accessory for modern smartphones</t>
         </is>
       </c>
-      <c r="K6" t="n">
-        <v>4990</v>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>10,000 mAh</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
           <t>10,000mAh capacity for reliable portable power.</t>
@@ -1184,6 +1543,7 @@
           <t>specs: manual-product-url (https://www.stuffcool.com/products/major-10000mah-20w-pd-powerbank) | mrp: input-sheet</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
           <t>ok</t>
@@ -1199,6 +1559,7 @@
           <t>10000mAh 20W PD powerbank with four charging ports</t>
         </is>
       </c>
+      <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr">
         <is>
           <t>10,000 mAh</t>
@@ -1244,6 +1605,8 @@
           <t>Four ports charge multiple devices at once.</t>
         </is>
       </c>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1254,6 +1617,40 @@
           <t>local-disk</t>
         </is>
       </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
+      <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1276,6 +1673,8 @@
           <t>https://www.stuffcool.com/products/roam-20000mah-mini-powerbank-with-20w-type-c-output</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>1499</v>
       </c>
@@ -1357,6 +1756,20 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1367,6 +1780,42 @@
           <t>brand-site</t>
         </is>
       </c>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/roam-20000mah-mini-powerbank-with-20w-type-c-output</t>
+        </is>
+      </c>
+      <c r="AU7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr"/>
+      <c r="BI7" t="inlineStr"/>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1384,6 +1833,9 @@
           <t>Odin</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>3199</v>
       </c>
@@ -1465,6 +1917,20 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1475,6 +1941,42 @@
           <t>brand-site</t>
         </is>
       </c>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/odin-10-000mah-qi2-magsafe-powerbank-with-built-in-type-c-cable</t>
+        </is>
+      </c>
+      <c r="AU8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr"/>
+      <c r="BI8" t="inlineStr"/>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr"/>
+      <c r="BQ8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1497,6 +1999,8 @@
           <t>https://www.stuffcool.com/products/1-22-5w-10000mah-powerbank-with-20w-pd-type-c-fast-charging</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>949</v>
       </c>
@@ -1538,6 +2042,7 @@
           <t>228gm</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
           <t>Charges compatible iPhones up to 50% in 30 minutes.</t>
@@ -1573,11 +2078,24 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
           <t>6 Months (Extendable to 1 Year)</t>
         </is>
       </c>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1588,6 +2106,42 @@
           <t>brand-site</t>
         </is>
       </c>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/1-22-5w-10000mah-powerbank-with-20w-pd-type-c-fast-charging</t>
+        </is>
+      </c>
+      <c r="AU9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
+      <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr"/>
+      <c r="BI9" t="inlineStr"/>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr"/>
+      <c r="BQ9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1610,6 +2164,8 @@
           <t>https://www.stuffcool.com/products/click-20000mah-15w-magnetic-wireless-powerbank-with-natural-titanium-finish-for-iphone</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>2375</v>
       </c>
@@ -1628,6 +2184,12 @@
           <t>Reliable &amp; durable charging accessory by Stuffcool</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
           <t>Reliable and durable brand quality from Stuffcool.</t>
@@ -1673,6 +2235,7 @@
           <t>20000mAh 15W magnetic wireless powerbank with digital display</t>
         </is>
       </c>
+      <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr">
         <is>
           <t>20,000 mAh / 77Wh</t>
@@ -1718,6 +2281,8 @@
           <t>Digital display shows exact battery percentage.</t>
         </is>
       </c>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1728,6 +2293,36 @@
           <t>amazon.in/dp/B0DFZ1KDPL</t>
         </is>
       </c>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="inlineStr"/>
+      <c r="BH10" t="inlineStr"/>
+      <c r="BI10" t="inlineStr"/>
+      <c r="BJ10" t="inlineStr"/>
+      <c r="BK10" t="inlineStr"/>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr"/>
+      <c r="BO10" t="inlineStr"/>
+      <c r="BP10" t="inlineStr"/>
+      <c r="BQ10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1745,6 +2340,9 @@
           <t>Omni pro</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>3799</v>
       </c>
@@ -1786,6 +2384,7 @@
           <t>214g ± 10g</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
           <t>25W Qi2.2 wireless fast charging for iPhone</t>
@@ -1821,11 +2420,24 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
           <t>6 Months (Extendable to 1 Year)</t>
         </is>
       </c>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1836,6 +2448,42 @@
           <t>brand-site</t>
         </is>
       </c>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>https://www.stuffcool.com/products/omni-pro-qi2-2-certified-25w-magsafe-powerbank-with-apple-watch-charger</t>
+        </is>
+      </c>
+      <c r="AU11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+      <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
+      <c r="BG11" t="inlineStr"/>
+      <c r="BH11" t="inlineStr"/>
+      <c r="BI11" t="inlineStr"/>
+      <c r="BJ11" t="inlineStr"/>
+      <c r="BK11" t="inlineStr"/>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="inlineStr"/>
+      <c r="BN11" t="inlineStr"/>
+      <c r="BO11" t="inlineStr"/>
+      <c r="BP11" t="inlineStr"/>
+      <c r="BQ11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: implement closed self-correction loop, vision fallback, auto-skip, partial specs policy, and brochure tier 0
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BQ11"/>
+  <dimension ref="A1:BQ31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2485,6 +2485,4049 @@
       <c r="BP11" t="inlineStr"/>
       <c r="BQ11" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PB-PEB-001</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Pebble PB Fuel</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>1375</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Pebble PB Fuel</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Reliable portable power bank with fast charging capabilities.</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>3499</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>22.5W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Type-C</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>6 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>10000 mAh total battery capacity for daily use.</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>22.5W Fast Charging output for rapid device power.</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Type-C port for universal device connection.</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>6 Months Warranty coverage for product assurance.</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/rapid-fuel)</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/0__1_c8d0b864-f557-4ba5-926e-dd491093756c.jpg?v=1765944792&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="AQ12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="AS12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="AU12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="AW12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="AY12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="BA12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="BE12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="BG12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="BI12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="BK12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
+      <c r="BM12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP12" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-PEB-001] Collected via tier-1: brand-page (https://www.pebblecart.com/products/rapid-fuel)</t>
+        </is>
+      </c>
+      <c r="BQ12" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PB-PEB-002</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Pebble PB Mag Mini 5K Black</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>950</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>Hard Block: All spec tiers exhausted without finding technical specifications</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="inlineStr"/>
+      <c r="BH13" t="inlineStr"/>
+      <c r="BI13" t="inlineStr"/>
+      <c r="BJ13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP13" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-PEB-002] BLOCKED: All tiers exhausted</t>
+        </is>
+      </c>
+      <c r="BQ13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PB-PEB-003</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pebble PB Rapid Air</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>900</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Pebble PB Rapid Air</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Compact 10000 mAh power bank featuring 22W fast charging and magnetic wireless.</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>2199</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>22W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Type-C, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>6 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity stores multiple device charges safely.</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>22W fast charging delivers high speed power output.</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>100g lightweight design ensures easy daily portability.</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>6 months warranty included against manufacturing defects.</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-rapid-air)</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/0__2_3c134667-4c49-4eeb-b07b-20b997440d66.jpg?v=1766126520&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>Rapid Air</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="AQ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="AS14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="AU14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="AW14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="AY14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="BA14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="BC14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="BE14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="BG14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="BI14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="BK14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL14" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
+        </is>
+      </c>
+      <c r="BM14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP14" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-PEB-003] Collected via tier-1: brand-page (https://www.pebblecart.com/products/pebble-rapid-air)</t>
+        </is>
+      </c>
+      <c r="BQ14" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PB-PEB-004</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>pebble PB rapid boost 65</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>2290</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>pebble PB rapid boost 65</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>High capacity power bank with fast charging capabilities and dual ports.</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>5499</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>20000 mAh</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>65W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Type-C, Built-in Type-C Cable</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>6 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>20000 mAh total power capacity for multiple device charges.</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>65W fast charging output delivers rapid power delivery.</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Type-C and built-in Type-C cable ports included.</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>6 months warranty included from the date of purchase.</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/rapid-boost-65) + tier-1-vision: brand-page (https://www.pebblecart.com/products/rapid-boost-65)</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/0_8190ee84-53c9-431c-958e-e0a4a84dbc3b.jpg?v=1769773990&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>Collected</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Rapid Boost 65</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="AQ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="AS15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="AU15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>1-vision</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="AY15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>1-vision</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="BE15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="BG15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="BI15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="BK15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL15" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
+        </is>
+      </c>
+      <c r="BM15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP15" t="inlineStr">
+        <is>
+          <t>Collected via tier-1: brand-page (https://www.pebblecart.com/products/rapid-boost-65) + tier-1-vision: brand-page (https://www.pebblecart.com/products/rapid-boost-65)</t>
+        </is>
+      </c>
+      <c r="BQ15" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PB-PEB-005</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pebble PB Rapid Electra 10</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>775</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>PB Rapid Electra 10</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Compact power bank equipped with multiple versatile charging ports.</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>1999</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>22.5W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>300g</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>6 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity stores backup power for devices.</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>22.5W fast charging delivers rapid power delivery.</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>300g lightweight build for everyday portability.</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>6 months warranty provides standard manufacturer support.</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-rapid-electra10)</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/0_5.jpg?v=1769772837&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Rapid Electra 10</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="AQ16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="AS16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="AU16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="AW16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="AY16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="BA16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="BC16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="BE16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="BG16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="BI16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="BK16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL16" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
+        </is>
+      </c>
+      <c r="BM16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP16" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-PEB-005] Collected via tier-1: brand-page (https://www.pebblecart.com/products/pebble-rapid-electra10)</t>
+        </is>
+      </c>
+      <c r="BQ16" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PB-PEB-006</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Pebble PB Rapid Electra 20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Pebble PB Rapid Electra 20</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>High capacity portable power bank equipped with multiple output ports.</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>3299</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>20000 mAh</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>22.5W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>6 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>20000 mAh capacity for multiple device charges.</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>22.5W fast charging output for rapid power delivery.</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Type-C and USB-A ports for versatile connections.</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>6 months warranty coverage for reliable support.</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-electra10)</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/1_07f09464-00cb-468f-a6a0-cd39a86108fc.jpg?v=1756367528&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>Rapid Electra 20</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="AQ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="AS17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="AU17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="AW17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="AY17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="BA17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="BC17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="BE17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="BG17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="BI17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="BK17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL17" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-electra10</t>
+        </is>
+      </c>
+      <c r="BM17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP17" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-PEB-006] Collected via tier-1: brand-page (https://www.pebblecart.com/products/pebble-electra10)</t>
+        </is>
+      </c>
+      <c r="BQ17" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PB-PEB-007</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pebble PB Rapid Nova 20</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>1475</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>PB Rapid Nova 20</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>High capacity portable power source with fast charging capabilities.</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>3499</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>20000 mAh</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>20W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Type-C</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>305g</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>6 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>20000 mAh capacity for extended mobile device usage.</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>20W fast charging output for rapid power delivery.</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Type-C port configuration for modern device connection.</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>305g total weight for portable everyday carrying.</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/rapid-nova20)</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/1_10647300-7d10-4e91-a9f4-27b9e1873fa7.jpg?v=1762766928&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>Rapid Nova 20</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="AQ18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="AS18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="AU18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="AW18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="AY18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="BA18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="BC18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="BE18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="BG18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="BI18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="BK18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL18" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-nova20</t>
+        </is>
+      </c>
+      <c r="BM18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP18" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-PEB-007] Collected via tier-1: brand-page (https://www.pebblecart.com/products/rapid-nova20)</t>
+        </is>
+      </c>
+      <c r="BQ18" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PB-POR-001</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Luxcell Mini</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>875</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>Hard Block: All spec tiers exhausted without finding technical specifications</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="n">
+        <v>2499</v>
+      </c>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr"/>
+      <c r="BH19" t="inlineStr"/>
+      <c r="BI19" t="inlineStr"/>
+      <c r="BJ19" t="inlineStr"/>
+      <c r="BK19" t="inlineStr"/>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="inlineStr"/>
+      <c r="BN19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP19" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-001] BLOCKED: All tiers exhausted</t>
+        </is>
+      </c>
+      <c r="BQ19" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PB-POR-002</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Luxcell Wireless Mini</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>1331</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Luxcell Wireless Mini</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Compact power bank featuring 10000 mAh capacity and magnetic wireless support.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>15W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity provides reliable emergency power.</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>15W fast charging delivers rapid device recovery.</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Magnetic wireless enables convenient cable-free charging.</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>12 months warranty ensures long-term dependability.</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.portronics.com/products/luxcell-wireless-mini-10k)</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/Luxcell_Wireless_Mini_10K_wireless_power_bank.jpg?v=1742981494&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr"/>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Wireless Mini</t>
+        </is>
+      </c>
+      <c r="AO20" t="n">
+        <v>3999</v>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="AQ20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="AS20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="AW20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="AY20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="BA20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB20" t="inlineStr"/>
+      <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="BE20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="BG20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="BI20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="BK20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL20" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
+        </is>
+      </c>
+      <c r="BM20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP20" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-002] Collected via tier-1: brand-page (https://www.portronics.com/products/luxcell-wireless-mini-10k)</t>
+        </is>
+      </c>
+      <c r="BQ20" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PB-POR-003</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Luxcell B12</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>599</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Portronics Luxcell B12</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Compact power bank equipped with multiple device charging ports.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>12W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity stores backup power for devices.</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>12W Fast Charging delivers quick power output.</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Type-C input allows standard cable connection.</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>12 Months Warranty provides official service cover.</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.portronics.com/products/luxcell-b12-type-c-input)</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/LuxcellB12_1.jpg?v=1785235352&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Luxcell B12</t>
+        </is>
+      </c>
+      <c r="AO21" t="n">
+        <v>3499</v>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="AQ21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="AS21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="AW21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="AY21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="BA21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB21" t="inlineStr"/>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="BE21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="BG21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="BI21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="BK21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL21" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
+        </is>
+      </c>
+      <c r="BM21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP21" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-003] Collected via tier-1: brand-page (https://www.portronics.com/products/luxcell-b12-type-c-input)</t>
+        </is>
+      </c>
+      <c r="BQ21" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PB-POR-004</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Power Shutter</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>1506</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Power Shutter</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Equipped with magnetic wireless capability and fast charging.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>15W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Type-C, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity provides reliable backup power.</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>15W fast charging delivers rapid device energy.</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Type-C and magnetic wireless ports offer charging.</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>12 months warranty ensures long-term product trust.</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.portronics.com/products/power-shutter)</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/Power_Shutter_wireless_power_bank_for.jpg?v=1730270085&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Power Shutter</t>
+        </is>
+      </c>
+      <c r="AO22" t="n">
+        <v>2499</v>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="AQ22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="AS22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr"/>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="AW22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="AY22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="BA22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB22" t="inlineStr"/>
+      <c r="BC22" t="inlineStr"/>
+      <c r="BD22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="BE22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="BG22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="BI22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="BK22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL22" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter</t>
+        </is>
+      </c>
+      <c r="BM22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP22" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-004] Collected via tier-1: brand-page (https://www.portronics.com/products/power-shutter)</t>
+        </is>
+      </c>
+      <c r="BQ22" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PB-POR-005</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Power Shutter Pro</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>1210</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Power Shutter Pro</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Portable power bank providing reliable device charging on the go.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>35W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity supports daily power needs.</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>35W fast charging output delivers rapid power.</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>12 months warranty provides manufacturer support.</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Compact design ensures easy everyday carry.</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>tier-2: brand-collection (https://www.portronics.com/products/power-shutter-pro)</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/Portronics_Power_Shutter_pro_10K_10000mah_powerbank_with_type_c_input.jpg?v=1731414090&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>Partial specifications: 2 of 5 specs empty (ports, weight)</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Shutter Pro</t>
+        </is>
+      </c>
+      <c r="AO23" t="n">
+        <v>3499</v>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="AQ23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="AS23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="AW23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="AY23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ23" t="inlineStr"/>
+      <c r="BA23" t="inlineStr"/>
+      <c r="BB23" t="inlineStr"/>
+      <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="BE23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="BG23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="BI23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BJ23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="BK23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL23" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-pro</t>
+        </is>
+      </c>
+      <c r="BM23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BN23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP23" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-005] Collected via tier-2: brand-collection (https://www.portronics.com/products/power-shutter-pro)</t>
+        </is>
+      </c>
+      <c r="BQ23" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PB-POR-006</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Chyro</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>1352</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Chyro Power Bank</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Compact portable charger with wireless and wired charging capabilities.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>15W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Type-C, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity for multiple device charges.</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>15W fast charging output for quick power delivery.</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Type-C and magnetic wireless ports included.</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>12 months warranty coverage for peace of mind.</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.portronics.com/products/chyro)</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/Chyro_10K_Power_Bank_10000mAh_Fast_Charging_Wireless_Power_Bank.jpg?v=1739515392&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr"/>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>Chyro</t>
+        </is>
+      </c>
+      <c r="AO24" t="n">
+        <v>2999</v>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="AQ24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="AS24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr"/>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="AW24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="AY24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="BA24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB24" t="inlineStr"/>
+      <c r="BC24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="BE24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="BG24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="BI24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="BK24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL24" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/chyro</t>
+        </is>
+      </c>
+      <c r="BM24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP24" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-006] Collected via tier-1: brand-page (https://www.portronics.com/products/chyro)</t>
+        </is>
+      </c>
+      <c r="BQ24" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PB-POR-007</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Power Shutter Air</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>1331</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Power Shutter Air</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Equipped with a 20000 mAh battery capacity and 15W fast charging.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>20000 mAh</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>15W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Type-C, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>20000 mAh capacity provides multiple device charges.</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>15W fast charging delivers rapid power delivery.</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Type-C and magnetic wireless ports offer versatile use.</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>12 months warranty ensures reliable long-term support.</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.portronics.com/products/power-shutter-air-20k)</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/portronics_power_shutter_air_20k_magnetic_wireless_power_bank.jpg?v=1786433087&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Shutter Air</t>
+        </is>
+      </c>
+      <c r="AO25" t="n">
+        <v>2999</v>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="AQ25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="AS25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT25" t="inlineStr"/>
+      <c r="AU25" t="inlineStr"/>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="AW25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="AY25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="BA25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB25" t="inlineStr"/>
+      <c r="BC25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="BE25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="BG25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="BI25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="BK25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL25" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
+        </is>
+      </c>
+      <c r="BM25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP25" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-007] Collected via tier-1: brand-page (https://www.portronics.com/products/power-shutter-air-20k)</t>
+        </is>
+      </c>
+      <c r="BQ25" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PB-POR-008</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Luxcell Stride</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>768</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>Hard Block: All spec tiers exhausted without finding technical specifications</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr"/>
+      <c r="AN26" t="inlineStr"/>
+      <c r="AO26" t="n">
+        <v>1999</v>
+      </c>
+      <c r="AP26" t="inlineStr"/>
+      <c r="AQ26" t="inlineStr"/>
+      <c r="AR26" t="inlineStr"/>
+      <c r="AS26" t="inlineStr"/>
+      <c r="AT26" t="inlineStr"/>
+      <c r="AU26" t="inlineStr"/>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr"/>
+      <c r="AX26" t="inlineStr"/>
+      <c r="AY26" t="inlineStr"/>
+      <c r="AZ26" t="inlineStr"/>
+      <c r="BA26" t="inlineStr"/>
+      <c r="BB26" t="inlineStr"/>
+      <c r="BC26" t="inlineStr"/>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="inlineStr"/>
+      <c r="BF26" t="inlineStr"/>
+      <c r="BG26" t="inlineStr"/>
+      <c r="BH26" t="inlineStr"/>
+      <c r="BI26" t="inlineStr"/>
+      <c r="BJ26" t="inlineStr"/>
+      <c r="BK26" t="inlineStr"/>
+      <c r="BL26" t="inlineStr"/>
+      <c r="BM26" t="inlineStr"/>
+      <c r="BN26" t="inlineStr"/>
+      <c r="BO26" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP26" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-008] BLOCKED: All tiers exhausted</t>
+        </is>
+      </c>
+      <c r="BQ26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PB-POR-009</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Luxcell UNO 10</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>768</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Luxcell UNO 10</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Compact power bank featuring high capacity and fast charging support.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>22.5W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>10000 mAh total capacity for multiple device charges.</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>22.5W Fast Charging output for rapid power delivery.</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Type-C and USB-A ports for versatile connectivity.</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>12 Months Warranty included for product assurance.</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.portronics.com/products/luxcell-uno-10)</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/Portronics_Luxcell_UNO_10K_Smallest_Power_Bank_Built-in_detachable_Type-C_cable.jpg?v=1763535396&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
+      <c r="AJ27" t="inlineStr"/>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>Luxcell UNO 10</t>
+        </is>
+      </c>
+      <c r="AO27" t="n">
+        <v>1999</v>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="AQ27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="AS27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT27" t="inlineStr"/>
+      <c r="AU27" t="inlineStr"/>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="AW27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="AY27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="BA27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB27" t="inlineStr"/>
+      <c r="BC27" t="inlineStr"/>
+      <c r="BD27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="BE27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="BG27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="BI27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="BK27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL27" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/luxcell-uno-10</t>
+        </is>
+      </c>
+      <c r="BM27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP27" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-009] Collected via tier-1: brand-page (https://www.portronics.com/products/luxcell-uno-10)</t>
+        </is>
+      </c>
+      <c r="BQ27" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PB-POR-010</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Revvo</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="n">
+        <v>1392</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Portronics Revvo</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Compact power bank featuring high capacity and fast wireless charging.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>15W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Type-C, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity for extended mobile device usage.</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>15W fast charging output delivers rapid power delivery.</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Type-C and magnetic wireless ports for dual charging.</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>12 months warranty included for long-term reliability.</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.portronics.com/products/revvo)</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/Portronics_Revvo_10000mAh_Magnetic_Wireless_Power_Bank.jpg?v=1762931528&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN28" t="inlineStr">
+        <is>
+          <t>Revvo</t>
+        </is>
+      </c>
+      <c r="AO28" t="n">
+        <v>2999</v>
+      </c>
+      <c r="AP28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="AQ28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="AS28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT28" t="inlineStr"/>
+      <c r="AU28" t="inlineStr"/>
+      <c r="AV28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="AW28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="AY28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="BA28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB28" t="inlineStr"/>
+      <c r="BC28" t="inlineStr"/>
+      <c r="BD28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="BE28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="BG28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="BI28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="BK28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL28" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/revvo</t>
+        </is>
+      </c>
+      <c r="BM28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP28" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-010] Collected via tier-1: brand-page (https://www.portronics.com/products/revvo)</t>
+        </is>
+      </c>
+      <c r="BQ28" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PB-POR-011</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Power Shutter</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>1506</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="inlineStr"/>
+      <c r="AI29" t="inlineStr"/>
+      <c r="AJ29" t="inlineStr"/>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>Hard Block: Duplicate image asset: identical file hash to product [PB-POR-004]</t>
+        </is>
+      </c>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN29" t="inlineStr"/>
+      <c r="AO29" t="n">
+        <v>2499</v>
+      </c>
+      <c r="AP29" t="inlineStr"/>
+      <c r="AQ29" t="inlineStr"/>
+      <c r="AR29" t="inlineStr"/>
+      <c r="AS29" t="inlineStr"/>
+      <c r="AT29" t="inlineStr"/>
+      <c r="AU29" t="inlineStr"/>
+      <c r="AV29" t="inlineStr"/>
+      <c r="AW29" t="inlineStr"/>
+      <c r="AX29" t="inlineStr"/>
+      <c r="AY29" t="inlineStr"/>
+      <c r="AZ29" t="inlineStr"/>
+      <c r="BA29" t="inlineStr"/>
+      <c r="BB29" t="inlineStr"/>
+      <c r="BC29" t="inlineStr"/>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="inlineStr"/>
+      <c r="BF29" t="inlineStr"/>
+      <c r="BG29" t="inlineStr"/>
+      <c r="BH29" t="inlineStr"/>
+      <c r="BI29" t="inlineStr"/>
+      <c r="BJ29" t="inlineStr"/>
+      <c r="BK29" t="inlineStr"/>
+      <c r="BL29" t="inlineStr"/>
+      <c r="BM29" t="inlineStr"/>
+      <c r="BN29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP29" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-011] Collected via tier-1: brand-page (https://www.portronics.com/products/power-shutter)
+Attempt 1: No automated fix available for flags: ['Duplicate image asset: identical file hash to product [PB-POR-004]']</t>
+        </is>
+      </c>
+      <c r="BQ29" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PB-POR-012</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Hally</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="n">
+        <v>1814</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr"/>
+      <c r="AJ30" t="inlineStr"/>
+      <c r="AK30" t="inlineStr">
+        <is>
+          <t>Hard Block: All spec tiers exhausted without finding technical specifications</t>
+        </is>
+      </c>
+      <c r="AL30" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="AM30" t="inlineStr"/>
+      <c r="AN30" t="inlineStr"/>
+      <c r="AO30" t="n">
+        <v>6999</v>
+      </c>
+      <c r="AP30" t="inlineStr"/>
+      <c r="AQ30" t="inlineStr"/>
+      <c r="AR30" t="inlineStr"/>
+      <c r="AS30" t="inlineStr"/>
+      <c r="AT30" t="inlineStr"/>
+      <c r="AU30" t="inlineStr"/>
+      <c r="AV30" t="inlineStr"/>
+      <c r="AW30" t="inlineStr"/>
+      <c r="AX30" t="inlineStr"/>
+      <c r="AY30" t="inlineStr"/>
+      <c r="AZ30" t="inlineStr"/>
+      <c r="BA30" t="inlineStr"/>
+      <c r="BB30" t="inlineStr"/>
+      <c r="BC30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr"/>
+      <c r="BE30" t="inlineStr"/>
+      <c r="BF30" t="inlineStr"/>
+      <c r="BG30" t="inlineStr"/>
+      <c r="BH30" t="inlineStr"/>
+      <c r="BI30" t="inlineStr"/>
+      <c r="BJ30" t="inlineStr"/>
+      <c r="BK30" t="inlineStr"/>
+      <c r="BL30" t="inlineStr"/>
+      <c r="BM30" t="inlineStr"/>
+      <c r="BN30" t="inlineStr"/>
+      <c r="BO30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP30" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-012] BLOCKED: All tiers exhausted</t>
+        </is>
+      </c>
+      <c r="BQ30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PB-POR-013</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Portronics</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Aero 65</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>1964</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Aero 65</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Portable power bank featuring 20000 mAh capacity and 65W fast charging.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>20000 mAh</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>65W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>12 Months Warranty</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>20000 mAh capacity provides multiple device charges.</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>65W fast charging delivers high speed power output.</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Type-C and USB-A ports enable dual device charging.</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>12 months warranty ensures long term reliability.</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.portronics.com/products/aero-65)</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/cdn/shop/files/Portronics_Aero_65_20000mAh_Power_Bank_at_best_price.jpg?v=1768387081&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
+      <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="inlineStr"/>
+      <c r="AI31" t="inlineStr"/>
+      <c r="AJ31" t="inlineStr"/>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>Aero 65</t>
+        </is>
+      </c>
+      <c r="AO31" t="n">
+        <v>3999</v>
+      </c>
+      <c r="AP31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="AQ31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="AS31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT31" t="inlineStr"/>
+      <c r="AU31" t="inlineStr"/>
+      <c r="AV31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="AW31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="AY31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="BA31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB31" t="inlineStr"/>
+      <c r="BC31" t="inlineStr"/>
+      <c r="BD31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="BE31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="BG31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="BI31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="BK31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL31" t="inlineStr">
+        <is>
+          <t>https://www.portronics.com/products/aero-65</t>
+        </is>
+      </c>
+      <c r="BM31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP31" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-POR-013] Collected via tier-1: brand-page (https://www.portronics.com/products/aero-65)</t>
+        </is>
+      </c>
+      <c r="BQ31" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Harden collection pipeline: 15s vision timeout, generic WooCommerce/Magento/custom parser, brand bot-block failover, remove dead Croma, multi-product brochure isolation, duplicate pre-flight, matcher regression tests, and resolve PB-URB-007 Arc
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BQ31"/>
+  <dimension ref="A1:BQ42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6528,6 +6528,2548 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PB-URB-001</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Nano 10000mAh 20W</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="n">
+        <v>1020</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Nano 10000mAh 20W Power Bank</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Compact power bank equipped with EV-grade lithium-ion cells and fast charging.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>20W Rocket Fast Charging</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Type-C</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity provides reliable mobile device power.</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>20W rocket fast charging output restores power quickly.</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1 type-c port handles both device charge and recharge.</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>1 year warranty is included for product protection.</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>tier-0-vision: (brochure: urbn_catalog.pdf, page 3)</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
+      <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr"/>
+      <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr"/>
+      <c r="AJ32" t="inlineStr"/>
+      <c r="AK32" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL32" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr">
+        <is>
+          <t>Nano</t>
+        </is>
+      </c>
+      <c r="AO32" t="inlineStr"/>
+      <c r="AP32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="AQ32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="AR32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="AS32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="AT32" t="inlineStr"/>
+      <c r="AU32" t="inlineStr"/>
+      <c r="AV32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="AW32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="AX32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="AY32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="AZ32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="BA32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="BB32" t="inlineStr"/>
+      <c r="BC32" t="inlineStr"/>
+      <c r="BD32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="BE32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="BF32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="BG32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="BH32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="BI32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="BJ32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="BK32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="BL32" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 3</t>
+        </is>
+      </c>
+      <c r="BM32" t="inlineStr">
+        <is>
+          <t>0-vision</t>
+        </is>
+      </c>
+      <c r="BN32" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO32" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP32" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-001] Collected via tier-0-vision: (brochure: urbn_catalog.pdf, page 3)</t>
+        </is>
+      </c>
+      <c r="BQ32" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PB-URB-002</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Atom Link MagSafe 10000mAh 20W</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>2125</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Atom Link MagSafe 10000mAh</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Compact power bank equipped with multiple charging output options.</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>6999</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>20W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>205g</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity provides reliable mobile power.</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>20W fast charging delivers rapid device recovery.</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>205g total weight offers portable everyday carry.</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, and magnetic wireless ports included.</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.urbnworld.com/products/10-000-mah-atom-link)</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>https://urbnworld.com/cdn/shop/files/1_8fee9d48-9539-4a7c-922c-beb272285777_1_compressed.webp?v=1754025165&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
+      <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr"/>
+      <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr"/>
+      <c r="AJ33" t="inlineStr"/>
+      <c r="AK33" t="inlineStr">
+        <is>
+          <t>URL slug numeric token mismatch: slug '10-000-mah-atom-link' contains numbers ['000', '10'] but title/model contains ['10000'] (potential reused URL handle)</t>
+        </is>
+      </c>
+      <c r="AL33" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN33" t="inlineStr">
+        <is>
+          <t>Atom Link</t>
+        </is>
+      </c>
+      <c r="AO33" t="inlineStr"/>
+      <c r="AP33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="AQ33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="AS33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="AU33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="AW33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="AY33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="BA33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="BC33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD33" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="BG33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="BI33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="BK33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL33" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
+        </is>
+      </c>
+      <c r="BM33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP33" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-002] Collected via tier-1: brand-page (https://www.urbnworld.com/products/10-000-mah-atom-link)</t>
+        </is>
+      </c>
+      <c r="BQ33" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PB-URB-003</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Frost MagSafe 10000mAh</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="n">
+        <v>1615</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Frost MagSafe 10000mAh</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Compact power bank featuring wireless and wired charging capabilities.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>15W</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Type-C</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>10000mAh capacity provides reliable backup power.</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>15W wireless output supports fast device charging.</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>20W wired output delivers rapid power delivery.</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Type-C input and output ensures broad connection.</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>tier-0: (brochure: urbn_catalog.pdf, page 13)</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr"/>
+      <c r="AF34" t="inlineStr"/>
+      <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="inlineStr"/>
+      <c r="AI34" t="inlineStr"/>
+      <c r="AJ34" t="inlineStr"/>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)
+Image is not square (1:1): 1200x1500px; tile is 290x290px square and will crop</t>
+        </is>
+      </c>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>Frost</t>
+        </is>
+      </c>
+      <c r="AO34" t="inlineStr"/>
+      <c r="AP34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="AQ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="AS34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT34" t="inlineStr"/>
+      <c r="AU34" t="inlineStr"/>
+      <c r="AV34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="AW34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="AY34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="BA34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB34" t="inlineStr"/>
+      <c r="BC34" t="inlineStr"/>
+      <c r="BD34" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="BG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="BI34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="BK34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL34" t="inlineStr">
+        <is>
+          <t>brochure: urbn_catalog.pdf, page 13</t>
+        </is>
+      </c>
+      <c r="BM34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN34" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO34" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP34" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-003] Collected via tier-0: (brochure: urbn_catalog.pdf, page 13)</t>
+        </is>
+      </c>
+      <c r="BQ34" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PB-URB-004</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Flux MagSafe Qi2 10000mAh</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="n">
+        <v>2550</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Flux MagSafe Qi2 10000mAh</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Compact magnetic wireless power bank with fast charging capabilities.</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>7999</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>22.5W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>234g</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity provides multiple device charges.</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>22.5W fast charging delivers rapid power output.</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>3 ports include Type-C, USB-A, and wireless.</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>234g lightweight design ensures easy portability.</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank)</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>https://urbnworld.com/cdn/shop/files/CopyofUPR116UrbnFluxMagTagPowerBankOnlineCatalogue-Dome01_195bf5b3-bf9f-4062-917d-e3a793245f3d.jpg?v=1779107514&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
+      <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr"/>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr"/>
+      <c r="AJ35" t="inlineStr"/>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>URL slug numeric token mismatch: slug '10-000mah-flux-qi2-magtag-power-bank' contains numbers ['000', '10', '2'] but title/model contains ['10000', '2'] (potential reused URL handle)</t>
+        </is>
+      </c>
+      <c r="AL35" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN35" t="inlineStr">
+        <is>
+          <t>Flux</t>
+        </is>
+      </c>
+      <c r="AO35" t="inlineStr"/>
+      <c r="AP35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AQ35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AS35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AU35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AW35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AY35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BA35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BC35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD35" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BG35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BI35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BK35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL35" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BM35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP35" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-004] Collected via tier-1: brand-page (https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank)</t>
+        </is>
+      </c>
+      <c r="BQ35" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PB-URB-005</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Slide Stand MagSafe 10000mAh</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="n">
+        <v>1530</v>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
+      <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
+      <c r="AF36" t="inlineStr"/>
+      <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr"/>
+      <c r="AJ36" t="inlineStr"/>
+      <c r="AK36" t="inlineStr">
+        <is>
+          <t>Skipped: Skipped: All spec tiers exhausted (including Vision) without finding technical specifications</t>
+        </is>
+      </c>
+      <c r="AL36" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="AM36" t="inlineStr"/>
+      <c r="AN36" t="inlineStr">
+        <is>
+          <t>Slide Stand</t>
+        </is>
+      </c>
+      <c r="AO36" t="inlineStr"/>
+      <c r="AP36" t="inlineStr"/>
+      <c r="AQ36" t="inlineStr"/>
+      <c r="AR36" t="inlineStr"/>
+      <c r="AS36" t="inlineStr"/>
+      <c r="AT36" t="inlineStr"/>
+      <c r="AU36" t="inlineStr"/>
+      <c r="AV36" t="inlineStr"/>
+      <c r="AW36" t="inlineStr"/>
+      <c r="AX36" t="inlineStr"/>
+      <c r="AY36" t="inlineStr"/>
+      <c r="AZ36" t="inlineStr"/>
+      <c r="BA36" t="inlineStr"/>
+      <c r="BB36" t="inlineStr"/>
+      <c r="BC36" t="inlineStr"/>
+      <c r="BD36" t="inlineStr"/>
+      <c r="BE36" t="inlineStr"/>
+      <c r="BF36" t="inlineStr"/>
+      <c r="BG36" t="inlineStr"/>
+      <c r="BH36" t="inlineStr"/>
+      <c r="BI36" t="inlineStr"/>
+      <c r="BJ36" t="inlineStr"/>
+      <c r="BK36" t="inlineStr"/>
+      <c r="BL36" t="inlineStr"/>
+      <c r="BM36" t="inlineStr"/>
+      <c r="BN36" t="inlineStr"/>
+      <c r="BO36" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP36" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-005] SKIPPED: All tiers exhausted</t>
+        </is>
+      </c>
+      <c r="BQ36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PB-URB-006</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Curve MagSafe 10000mAh</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="n">
+        <v>1530</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Curve MagSafe 10000mAh</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Compact power bank equipped with multiple output options and magnetic wireless.</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>4999</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>20W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>195g</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>10000 mAh total capacity for daily device charging needs.</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>20W fast charging output via wired connection ports.</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>3 versatile charging ports include Type-C and USB-A.</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>195g total weight designed for portable daily carry.</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank)</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>https://urbnworld.com/cdn/shop/files/UPR121_Curve_3-in-1_Magtag_Powerbank_online_catalogue-1.jpg?v=1776409442&amp;width={width}</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
+      <c r="AD37" t="inlineStr"/>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr"/>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr"/>
+      <c r="AJ37" t="inlineStr"/>
+      <c r="AK37" t="inlineStr"/>
+      <c r="AL37" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM37" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN37" t="inlineStr">
+        <is>
+          <t>Curve</t>
+        </is>
+      </c>
+      <c r="AO37" t="inlineStr"/>
+      <c r="AP37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="AQ37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="AS37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="AU37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="AW37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="AY37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="BA37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="BC37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD37" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="BG37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="BI37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="BK37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL37" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
+        </is>
+      </c>
+      <c r="BM37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP37" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-006] Collected via tier-1: brand-page (https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank)</t>
+        </is>
+      </c>
+      <c r="BQ37" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PB-URB-007</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Arc MagSafe 10000mAh</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="n">
+        <v>1275</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Arc MagSafe 10000mAh</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Magnetic wireless power bank with integrated stand and pass-through charging.</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>2999</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>15W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>220g</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity with built-in Li-Polymer battery cells.</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>15W wireless charging and 20W wired power delivery output.</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>12 layers of protection ensuring safe daily device usage.</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>6 months manufacturer warranty included with purchase.</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank) + tier-3: retail-reliance (https://www.reliancedigital.in/product/urbn-10000-mah-15-w-arc-magtag-power-bank-with-stand-black-mgp5oz-9546389)</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>https://urbnworld.com/cdn/shop/files/UPR123_BK_7_11zon.jpg?v=1749790783&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
+      <c r="AD38" t="inlineStr"/>
+      <c r="AE38" t="inlineStr"/>
+      <c r="AF38" t="inlineStr"/>
+      <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="inlineStr"/>
+      <c r="AI38" t="inlineStr"/>
+      <c r="AJ38" t="inlineStr"/>
+      <c r="AK38" t="inlineStr"/>
+      <c r="AL38" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN38" t="inlineStr">
+        <is>
+          <t>Arc</t>
+        </is>
+      </c>
+      <c r="AO38" t="inlineStr"/>
+      <c r="AP38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AQ38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AS38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AU38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AW38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX38" t="inlineStr">
+        <is>
+          <t>https://www.reliancedigital.in/product/urbn-10000-mah-15-w-arc-magtag-power-bank-with-stand-black-mgp5oz-9546389</t>
+        </is>
+      </c>
+      <c r="AY38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ38" t="inlineStr">
+        <is>
+          <t>https://www.reliancedigital.in/product/urbn-10000-mah-15-w-arc-magtag-power-bank-with-stand-black-mgp5oz-9546389</t>
+        </is>
+      </c>
+      <c r="BA38" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB38" t="inlineStr">
+        <is>
+          <t>https://www.reliancedigital.in/product/urbn-10000-mah-15-w-arc-magtag-power-bank-with-stand-black-mgp5oz-9546389</t>
+        </is>
+      </c>
+      <c r="BC38" t="n">
+        <v>3</v>
+      </c>
+      <c r="BD38" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BG38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BI38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BK38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL38" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BM38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP38" t="inlineStr">
+        <is>
+          <t>Collected via tier-1: brand-page (https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank) + tier-3: retail-reliance (https://www.reliancedigital.in/product/urbn-10000-mah-15-w-arc-magtag-power-bank-with-stand-black-mgp5oz-9546389)</t>
+        </is>
+      </c>
+      <c r="BQ38" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PB-URB-008</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Mini-Volt 10000mAh 35W</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="n">
+        <v>1760</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Mini-Volt 10000mAh 35W</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Compact power bank featuring dual output ports for rapid device charging.</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>2999</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>35W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>180g</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity stores multiple full charges.</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>35W fast charging delivers rapid power output.</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Type-C and USB-A ports support dual devices.</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>180g lightweight build offers easy portability.</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank)</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>https://urbnworld.com/cdn/shop/files/Artboard1_4fb97e0a-6b3c-4426-ba2b-d3cecb6d695d.webp?v=1767943682&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
+      <c r="Z39" t="inlineStr"/>
+      <c r="AA39" t="inlineStr"/>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
+      <c r="AD39" t="inlineStr"/>
+      <c r="AE39" t="inlineStr"/>
+      <c r="AF39" t="inlineStr"/>
+      <c r="AG39" t="inlineStr"/>
+      <c r="AH39" t="inlineStr"/>
+      <c r="AI39" t="inlineStr"/>
+      <c r="AJ39" t="inlineStr"/>
+      <c r="AK39" t="inlineStr">
+        <is>
+          <t>URL slug numeric token mismatch: slug '10-000mah-mini-volt-35w-power-bank' contains numbers ['000', '10', '35'] but title/model contains ['10000', '35'] (potential reused URL handle)</t>
+        </is>
+      </c>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN39" t="inlineStr">
+        <is>
+          <t>Mini-Volt</t>
+        </is>
+      </c>
+      <c r="AO39" t="inlineStr"/>
+      <c r="AP39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="AQ39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="AS39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="AU39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="AW39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="AY39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="BA39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="BC39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD39" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="BG39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="BI39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="BK39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL39" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
+        </is>
+      </c>
+      <c r="BM39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP39" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-008] Collected via tier-1: brand-page (https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank)</t>
+        </is>
+      </c>
+      <c r="BQ39" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PB-URB-009</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Aero Mag Tag 10000mAh</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>1680</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Aero Mag Tag 10000mAh</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Magnetic wireless power bank with 10000mAh capacity and 20W fast charging.</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>3999</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>20W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>194g</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>10000mAh capacity provides multiple full device charges.</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>20W fast charging delivers rapid power delivery speeds.</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>194g lightweight design ensures easy daily portability.</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, and magnetic wireless connection ports.</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank)</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>https://urbnworld.com/cdn/shop/files/Artboard_1_copy.webp?v=1766128181&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr"/>
+      <c r="AA40" t="inlineStr"/>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
+      <c r="AD40" t="inlineStr"/>
+      <c r="AE40" t="inlineStr"/>
+      <c r="AF40" t="inlineStr"/>
+      <c r="AG40" t="inlineStr"/>
+      <c r="AH40" t="inlineStr"/>
+      <c r="AI40" t="inlineStr"/>
+      <c r="AJ40" t="inlineStr"/>
+      <c r="AK40" t="inlineStr">
+        <is>
+          <t>URL slug numeric token mismatch: slug '10-000-mah-aero-magtag-power-bank' contains numbers ['000', '10'] but title/model contains ['10000'] (potential reused URL handle)</t>
+        </is>
+      </c>
+      <c r="AL40" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM40" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN40" t="inlineStr">
+        <is>
+          <t>Aero Mag Tag</t>
+        </is>
+      </c>
+      <c r="AO40" t="inlineStr"/>
+      <c r="AP40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AQ40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AS40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AU40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AW40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AY40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BA40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BC40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD40" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BG40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BI40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BK40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL40" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BM40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP40" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-009] Collected via tier-1: brand-page (https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank)</t>
+        </is>
+      </c>
+      <c r="BQ40" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PB-URB-010</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Slate MagSafe Qi2 10000mAh</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="n">
+        <v>2125</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Slate MagSafe Qi2 10000mAh</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Compact 10000mAh magnetic wireless power bank with 20W fast charging output.</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>4999</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>20W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>200g</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity provides reliable mobile backup power.</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>20W fast charging delivers rapid power delivery speeds.</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>200g lightweight design ensures easy daily portability.</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, and magnetic wireless charging ports.</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank)</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>https://urbnworld.com/cdn/shop/files/CopyofUPR129-10_000mAhSlateMagTagPowerBankonlinecatalogue-Dome01.jpg?v=1779103079&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr"/>
+      <c r="Y41" t="inlineStr"/>
+      <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
+      <c r="AD41" t="inlineStr"/>
+      <c r="AE41" t="inlineStr"/>
+      <c r="AF41" t="inlineStr"/>
+      <c r="AG41" t="inlineStr"/>
+      <c r="AH41" t="inlineStr"/>
+      <c r="AI41" t="inlineStr"/>
+      <c r="AJ41" t="inlineStr"/>
+      <c r="AK41" t="inlineStr">
+        <is>
+          <t>URL slug numeric token mismatch: slug '10-000mah-slate-qi2-magtag-power-bank' contains numbers ['000', '10', '2'] but title/model contains ['10000', '2'] (potential reused URL handle)</t>
+        </is>
+      </c>
+      <c r="AL41" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN41" t="inlineStr">
+        <is>
+          <t>Slate</t>
+        </is>
+      </c>
+      <c r="AO41" t="inlineStr"/>
+      <c r="AP41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AQ41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AS41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AU41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AW41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="AY41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BA41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BC41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD41" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BG41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BI41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BK41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL41" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
+        </is>
+      </c>
+      <c r="BM41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP41" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-010] Collected via tier-1: brand-page (https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank)</t>
+        </is>
+      </c>
+      <c r="BQ41" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PB-URB-011</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Urbn</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Ultra-Volt 20000mAh 65W</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="n">
+        <v>2800</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Ultra-Volt 20000mAh</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>High capacity portable charger with dual charging ports and fast output.</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>4999</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>20000 mAh</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>70W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>343g</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>20000 mAh capacity stores multiple full device charges.</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>70W Fast Charging delivers high speed power delivery.</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Type-C and USB-A ports support versatile connection.</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>343g weight offers portable travel convenience.</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.urbnworld.com/products/20-000mah-ultra-volt-65w)</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>https://urbnworld.com/cdn/shop/files/20_000mAh_Ultra_Volt_70W_online_catalogue-01.webp?v=1785324708&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr"/>
+      <c r="Y42" t="inlineStr"/>
+      <c r="Z42" t="inlineStr"/>
+      <c r="AA42" t="inlineStr"/>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
+      <c r="AD42" t="inlineStr"/>
+      <c r="AE42" t="inlineStr"/>
+      <c r="AF42" t="inlineStr"/>
+      <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr"/>
+      <c r="AJ42" t="inlineStr"/>
+      <c r="AK42" t="inlineStr">
+        <is>
+          <t>URL slug numeric token mismatch: slug '20-000mah-ultra-volt-65w' contains numbers ['000', '20', '65'] but title/model contains ['20000'] (potential reused URL handle)</t>
+        </is>
+      </c>
+      <c r="AL42" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AM42" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN42" t="inlineStr">
+        <is>
+          <t>Ultra-Volt</t>
+        </is>
+      </c>
+      <c r="AO42" t="inlineStr"/>
+      <c r="AP42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="AQ42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="AS42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="AU42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="AW42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="AY42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="BA42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="BC42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD42" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="BG42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="BI42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="BK42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL42" t="inlineStr">
+        <is>
+          <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
+        </is>
+      </c>
+      <c r="BM42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP42" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-URB-011] Collected via tier-1: brand-page (https://www.urbnworld.com/products/20-000mah-ultra-volt-65w)</t>
+        </is>
+      </c>
+      <c r="BQ42" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Implement Step 5.5: Automatic post-run LLM review, auto-recollection, Display_Name sanitization, and single table presentation
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -6760,7 +6760,7 @@
         <v>1</v>
       </c>
       <c r="BO32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP32" t="inlineStr">
         <is>
@@ -7007,7 +7007,7 @@
         <v>1</v>
       </c>
       <c r="BO33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP33" t="inlineStr">
         <is>
@@ -7233,7 +7233,7 @@
         <v>1</v>
       </c>
       <c r="BO34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP34" t="inlineStr">
         <is>
@@ -7480,7 +7480,7 @@
         <v>1</v>
       </c>
       <c r="BO35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP35" t="inlineStr">
         <is>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="AM37" t="inlineStr">
         <is>
-          <t>brand-product-page</t>
+          <t>local-verified</t>
         </is>
       </c>
       <c r="AN37" t="inlineStr">
@@ -7826,7 +7826,7 @@
         <v>1</v>
       </c>
       <c r="BO37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP37" t="inlineStr">
         <is>
@@ -8069,7 +8069,7 @@
         <v>1</v>
       </c>
       <c r="BO38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP38" t="inlineStr">
         <is>
@@ -8207,7 +8207,7 @@
       </c>
       <c r="AM39" t="inlineStr">
         <is>
-          <t>brand-product-page</t>
+          <t>local-verified</t>
         </is>
       </c>
       <c r="AN39" t="inlineStr">
@@ -8316,7 +8316,7 @@
         <v>1</v>
       </c>
       <c r="BO39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP39" t="inlineStr">
         <is>
@@ -8454,7 +8454,7 @@
       </c>
       <c r="AM40" t="inlineStr">
         <is>
-          <t>brand-product-page</t>
+          <t>local-verified</t>
         </is>
       </c>
       <c r="AN40" t="inlineStr">
@@ -8563,7 +8563,7 @@
         <v>1</v>
       </c>
       <c r="BO40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP40" t="inlineStr">
         <is>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="AM41" t="inlineStr">
         <is>
-          <t>brand-product-page</t>
+          <t>local-verified</t>
         </is>
       </c>
       <c r="AN41" t="inlineStr">
@@ -8810,7 +8810,7 @@
         <v>1</v>
       </c>
       <c r="BO41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP41" t="inlineStr">
         <is>
@@ -8948,7 +8948,7 @@
       </c>
       <c r="AM42" t="inlineStr">
         <is>
-          <t>brand-product-page</t>
+          <t>local-verified</t>
         </is>
       </c>
       <c r="AN42" t="inlineStr">
@@ -9057,7 +9057,7 @@
         <v>1</v>
       </c>
       <c r="BO42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Approve Urbn products and append Urbn to combined catalogue PDF (23 pages)
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -6638,7 +6638,7 @@
       </c>
       <c r="AL32" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM32" t="inlineStr">
@@ -6893,7 +6893,7 @@
       </c>
       <c r="AL33" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM33" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="AL34" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM34" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="AL35" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM35" t="inlineStr">
@@ -7712,7 +7712,7 @@
       <c r="AK37" t="inlineStr"/>
       <c r="AL37" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM37" t="inlineStr">
@@ -7955,7 +7955,7 @@
       <c r="AK38" t="inlineStr"/>
       <c r="AL38" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM38" t="inlineStr">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="AL39" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM39" t="inlineStr">
@@ -8449,7 +8449,7 @@
       </c>
       <c r="AL40" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM40" t="inlineStr">
@@ -8696,7 +8696,7 @@
       </c>
       <c r="AL41" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM41" t="inlineStr">
@@ -8943,7 +8943,7 @@
       </c>
       <c r="AL42" t="inlineStr">
         <is>
-          <t>Ready_For_Review</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="AM42" t="inlineStr">

</xml_diff>

<commit_message>
Onboard brand EVM: 5/5 products approved, studio packshots verified, appended to combined catalogue
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BQ42"/>
+  <dimension ref="A1:BQ47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9070,6 +9070,1189 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PB-EVM-001</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>EVM</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Encharge</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="n">
+        <v>468</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Encharge</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Reliable mobile power supply for all corporate communication needs.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>10W Output</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Type-C, Micro-USB</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>10000mAh capacity provides reliable backup power.</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>10W output ensures efficient device charging.</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Type-C and Micro-USB ports offer dual input.</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>2 years manufacture warranty included for users.</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://evmzone.com/evm-products/encharge.html)</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/pub/media/catalog/product/0/1/01_2.jpg</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr"/>
+      <c r="Y43" t="inlineStr"/>
+      <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr"/>
+      <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
+      <c r="AF43" t="inlineStr"/>
+      <c r="AG43" t="inlineStr"/>
+      <c r="AH43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr"/>
+      <c r="AJ43" t="inlineStr"/>
+      <c r="AK43" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL43" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN43" t="inlineStr">
+        <is>
+          <t>Encharge</t>
+        </is>
+      </c>
+      <c r="AO43" t="n">
+        <v>1649</v>
+      </c>
+      <c r="AP43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="AQ43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="AS43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT43" t="inlineStr"/>
+      <c r="AU43" t="inlineStr"/>
+      <c r="AV43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="AW43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="AY43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="BA43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB43" t="inlineStr"/>
+      <c r="BC43" t="inlineStr"/>
+      <c r="BD43" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="BG43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="BI43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="BK43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL43" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/encharge.html</t>
+        </is>
+      </c>
+      <c r="BM43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP43" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-EVM-001] Collected via tier-1: brand-page (https://evmzone.com/evm-products/encharge.html)
+Attempt 1: No automated fix available for flags: ['Insufficient specifications: 3 of 5 required specs are empty (fewer than 3 populated)']
+Attempt 1: [PB-EVM-001] Collected via tier-1: brand-page (https://evmzone.com/evm-products/encharge.html)</t>
+        </is>
+      </c>
+      <c r="BQ43" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PB-EVM-002</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>EVM</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Enbolt</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="n">
+        <v>540</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>EVM Enbolt Power Bank</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Compact power source featuring high capacity and fast output delivery.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>22.5W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Micro-USB</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity for multiple device charges.</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>22.5W fast charging output reduces waiting times.</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>3 versatile ports include Type-C, USB-A and Micro.</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Type-C port supports modern device connections.</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html) + tier-1-vision: brand-page (https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html)</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/pub/media/catalog/product/0/1/01_264_5.jpg</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr"/>
+      <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr"/>
+      <c r="AD44" t="inlineStr"/>
+      <c r="AE44" t="inlineStr"/>
+      <c r="AF44" t="inlineStr"/>
+      <c r="AG44" t="inlineStr"/>
+      <c r="AH44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr"/>
+      <c r="AJ44" t="inlineStr"/>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL44" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN44" t="inlineStr">
+        <is>
+          <t>Enbolt</t>
+        </is>
+      </c>
+      <c r="AO44" t="n">
+        <v>2399</v>
+      </c>
+      <c r="AP44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="AQ44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="AS44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT44" t="inlineStr"/>
+      <c r="AU44" t="inlineStr"/>
+      <c r="AV44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="AW44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="AY44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="BA44" t="inlineStr">
+        <is>
+          <t>1-vision</t>
+        </is>
+      </c>
+      <c r="BB44" t="inlineStr"/>
+      <c r="BC44" t="inlineStr"/>
+      <c r="BD44" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE44" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="BG44" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="BI44" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="BK44" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL44" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
+        </is>
+      </c>
+      <c r="BM44" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN44" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO44" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP44" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-EVM-002] Collected via tier-1: brand-page (https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html) + tier-1-vision: brand-page (https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html)</t>
+        </is>
+      </c>
+      <c r="BQ44" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PB-EVM-003</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>EVM</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>EnMag Ace</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="n">
+        <v>900</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>EnMag Ace Power Bank</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Compact magnetic wireless power solution for daily charging.</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>15W Fast Charging</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity supports extended power needs.</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>15W fast charging delivers rapid device power.</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Type-C port provides reliable wired connection.</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Magnetic wireless allows cable-free charging.</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://evmzone.com/enmag-ace-power-bank-evm-p0301.html)</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/pub/media/catalog/product/e/n/enmag_ace_a_black_image_1.jpg</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr"/>
+      <c r="AD45" t="inlineStr"/>
+      <c r="AE45" t="inlineStr"/>
+      <c r="AF45" t="inlineStr"/>
+      <c r="AG45" t="inlineStr"/>
+      <c r="AH45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr"/>
+      <c r="AJ45" t="inlineStr"/>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr">
+        <is>
+          <t>EnMag Ace</t>
+        </is>
+      </c>
+      <c r="AO45" t="n">
+        <v>3999</v>
+      </c>
+      <c r="AP45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="AQ45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="AS45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT45" t="inlineStr"/>
+      <c r="AU45" t="inlineStr"/>
+      <c r="AV45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="AW45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="AY45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="BA45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB45" t="inlineStr"/>
+      <c r="BC45" t="inlineStr"/>
+      <c r="BD45" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="BG45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="BI45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="BK45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL45" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
+        </is>
+      </c>
+      <c r="BM45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP45" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-EVM-003] Collected via tier-1: brand-page (https://evmzone.com/enmag-ace-power-bank-evm-p0301.html)
+Attempt 1: No automated fix available for flags: ['Insufficient specifications: 3 of 5 required specs are empty (fewer than 3 populated)']
+Attempt 1: [PB-EVM-003] Collected via tier-1: brand-page (https://evmzone.com/enmag-ace-power-bank-evm-p0301.html)</t>
+        </is>
+      </c>
+      <c r="BQ45" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PB-EVM-004</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>EVM</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Enwire</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="n">
+        <v>695</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>EVM Enwire Power Bank</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Reliable portable charging solution equipped with an integrated 4-in-1 cable.</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>10W Output</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Micro-USB, Lightning</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>2 Years Warranty</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>10000mAh capacity provides backup power for mobile devices.</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>5 to 6 hours charge time for complete power restoration.</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>2.4 Amp output delivers fast charging capabilities.</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>2 years warranty included from the date of purchase.</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://evmzone.com/evm-products/powerbank/encase-power-bank.html)</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/pub/media/catalog/product/e/n/encase_power_bank_14_.jpg</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr"/>
+      <c r="Y46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr"/>
+      <c r="AA46" t="inlineStr"/>
+      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr"/>
+      <c r="AD46" t="inlineStr"/>
+      <c r="AE46" t="inlineStr"/>
+      <c r="AF46" t="inlineStr"/>
+      <c r="AG46" t="inlineStr"/>
+      <c r="AH46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr"/>
+      <c r="AJ46" t="inlineStr"/>
+      <c r="AK46" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL46" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN46" t="inlineStr">
+        <is>
+          <t>Enwire</t>
+        </is>
+      </c>
+      <c r="AO46" t="n">
+        <v>2700</v>
+      </c>
+      <c r="AP46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="AQ46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="AS46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT46" t="inlineStr"/>
+      <c r="AU46" t="inlineStr"/>
+      <c r="AV46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="AW46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="AY46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="BA46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB46" t="inlineStr"/>
+      <c r="BC46" t="inlineStr"/>
+      <c r="BD46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="BE46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="BG46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="BI46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="BK46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL46" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
+        </is>
+      </c>
+      <c r="BM46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP46" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-EVM-004] SKIPPED: All tiers exhausted
+Attempt 1: [PB-EVM-004] Collected via tier-1: brand-page (https://evmzone.com/evm-products/powerbank/encase-power-bank.html)</t>
+        </is>
+      </c>
+      <c r="BQ46" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PB-EVM-005</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>EVM</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Enwing</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="n">
+        <v>440</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Enwing EnMove Power Bank</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Portable 10000mAh backup power solution with dual USB ports and LED indicators.</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>12W Output</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Type-C, Micro-USB</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>10000mAh Li-polymer battery capacity for daily use.</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>12W Output delivers efficient multi-device charging.</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>2 USB ports enable simultaneous device charging.</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>5V/2.4A current output provides steady charging.</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://evmzone.com/evm-products/powerbank/enmove.html)</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/pub/media/catalog/product/0/1/01_13.jpg</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
+      <c r="AD47" t="inlineStr"/>
+      <c r="AE47" t="inlineStr"/>
+      <c r="AF47" t="inlineStr"/>
+      <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="inlineStr"/>
+      <c r="AI47" t="inlineStr"/>
+      <c r="AJ47" t="inlineStr"/>
+      <c r="AK47" t="inlineStr">
+        <is>
+          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+        </is>
+      </c>
+      <c r="AL47" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AN47" t="inlineStr">
+        <is>
+          <t>Enwing</t>
+        </is>
+      </c>
+      <c r="AO47" t="n">
+        <v>1999</v>
+      </c>
+      <c r="AP47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="AQ47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="AS47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT47" t="inlineStr"/>
+      <c r="AU47" t="inlineStr"/>
+      <c r="AV47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="AW47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="AY47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="BA47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB47" t="inlineStr"/>
+      <c r="BC47" t="inlineStr"/>
+      <c r="BD47" t="inlineStr">
+        <is>
+          <t>brand-default-policy</t>
+        </is>
+      </c>
+      <c r="BE47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="BG47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="BI47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="BK47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL47" t="inlineStr">
+        <is>
+          <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
+        </is>
+      </c>
+      <c r="BM47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP47" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-EVM-005] SKIPPED: All tiers exhausted
+Attempt 1: [PB-EVM-005] Collected via tier-1: brand-page (https://evmzone.com/evm-products/powerbank/enmove.html)</t>
+        </is>
+      </c>
+      <c r="BQ47" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Phase 0: Foundation API layer with SQLite job store, atomic single worker, brand lock, and progress callbacks
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -2845,7 +2845,11 @@
         </is>
       </c>
       <c r="AN13" t="inlineStr"/>
-      <c r="AO13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="inlineStr"/>
@@ -2877,7 +2881,8 @@
       </c>
       <c r="BQ13" t="inlineStr">
         <is>
-          <t>Attempt 1: [PB-PEB-002] BLOCKED: All tiers exhausted</t>
+          <t>Attempt 1: [PB-PEB-002] BLOCKED: All tiers exhausted
+Cleaned Display_Name to 'nan'</t>
         </is>
       </c>
       <c r="BR13" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix 2: Add Override_DP and separate DP and MRP override resolution chains
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR47"/>
+  <dimension ref="A1:BS47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -765,6 +765,11 @@
       <c r="BR1" t="inlineStr">
         <is>
           <t>LLM_Provider</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>Override_DP</t>
         </is>
       </c>
     </row>
@@ -933,6 +938,7 @@
       <c r="BP2" t="inlineStr"/>
       <c r="BQ2" t="inlineStr"/>
       <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1099,6 +1105,7 @@
       <c r="BP3" t="inlineStr"/>
       <c r="BQ3" t="inlineStr"/>
       <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1301,6 +1308,7 @@
       <c r="BP4" t="inlineStr"/>
       <c r="BQ4" t="inlineStr"/>
       <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1491,6 +1499,7 @@
       <c r="BP5" t="inlineStr"/>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1681,6 +1690,7 @@
       <c r="BP6" t="inlineStr"/>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1851,6 +1861,7 @@
       <c r="BP7" t="inlineStr"/>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2017,6 +2028,7 @@
       <c r="BP8" t="inlineStr"/>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2187,6 +2199,7 @@
       <c r="BP9" t="inlineStr"/>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2373,6 +2386,7 @@
       <c r="BP10" t="inlineStr"/>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2539,6 +2553,7 @@
       <c r="BP11" t="inlineStr"/>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2777,6 +2792,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2845,11 +2861,7 @@
         </is>
       </c>
       <c r="AN13" t="inlineStr"/>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="inlineStr"/>
@@ -2886,6 +2898,7 @@
         </is>
       </c>
       <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3134,6 +3147,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3376,6 +3390,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3624,6 +3639,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3872,6 +3888,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4120,6 +4137,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4240,6 +4258,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4476,6 +4495,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4712,6 +4732,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4948,6 +4969,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5174,6 +5196,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5410,6 +5433,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5646,6 +5670,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5752,6 +5777,7 @@
         </is>
       </c>
       <c r="BR26" t="inlineStr"/>
+      <c r="BS26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5988,6 +6014,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6224,6 +6251,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6345,6 +6373,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6451,6 +6480,7 @@
         </is>
       </c>
       <c r="BR30" t="inlineStr"/>
+      <c r="BS30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6687,6 +6717,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6937,6 +6968,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7189,6 +7221,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7420,6 +7453,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7672,6 +7706,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7780,6 +7815,7 @@
         </is>
       </c>
       <c r="BR36" t="inlineStr"/>
+      <c r="BS36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8028,6 +8064,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8276,6 +8313,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8528,6 +8566,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8780,6 +8819,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9032,6 +9072,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9284,6 +9325,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9526,6 +9568,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9768,6 +9811,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -10010,6 +10054,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -10251,6 +10296,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -10492,6 +10538,7 @@
           <t>gemini</t>
         </is>
       </c>
+      <c r="BS47" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix: Ensure display_name and clean card title overrides render seamlessly in catalogue build
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -1202,7 +1202,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Stuffcool Giga 20000mAh Powerbank</t>
+          <t>Giga</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Stuffcool Lucid 5000mAh Powerbank</t>
+          <t>Lucid</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Stuffcool Major 10000mAh Powerbank</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Stuffcool Click 20 Powerbank</t>
+          <t>Click 20</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">

</xml_diff>

<commit_message>
fix(pipeline): decouple specs and images, add image gate fallback, smart 2-pass brochure scanner, and Stage 2 price parsing
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS47"/>
+  <dimension ref="A1:BS49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -838,11 +838,7 @@
           <t>181g ± 10g</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 1 Year)</t>
-        </is>
-      </c>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>10,000mAh capacity with a stylish gold finish</t>
@@ -1005,11 +1001,7 @@
           <t>186g ± 10g</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>6 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>15W magnetic wireless charging for iPhone 12 and above.</t>
@@ -1231,11 +1223,7 @@
           <t>380g (10.8 x 6.8 x 3.25 cm)</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 1 Year)</t>
-        </is>
-      </c>
+      <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr">
         <is>
           <t>Built-in 65W Type-C cable charges MacBooks and laptops.</t>
@@ -1426,11 +1414,7 @@
           <t>105g ± 10g (7.7 x 6.6 x 2.05 cm)</t>
         </is>
       </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 1 Year)</t>
-        </is>
-      </c>
+      <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr">
         <is>
           <t>Smallest 5000mAh magnetic wireless powerbank.</t>
@@ -1619,11 +1603,7 @@
           <t>230g (14 x 6.8 x 1.74 cm)</t>
         </is>
       </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 1 Year)</t>
-        </is>
-      </c>
+      <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr">
         <is>
           <t>10,000mAh slim powerbank, proudly Made in India.</t>
@@ -1761,11 +1741,7 @@
           <t>322g ± 10g</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 1 Year)</t>
-        </is>
-      </c>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
           <t>20,000mAh capacity in an ultra-compact travel design</t>
@@ -1928,11 +1904,7 @@
           <t>230g ± 10g</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 12 Months)</t>
-        </is>
-      </c>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>15W Qi2 MagSafe fast wireless charging for iPhones.</t>
@@ -2142,11 +2114,7 @@
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 1 Year)</t>
-        </is>
-      </c>
+      <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
@@ -2319,11 +2287,7 @@
           <t>326g ± 10g (11.0 x 6.9 x 2.85 cm)</t>
         </is>
       </c>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 1 Year)</t>
-        </is>
-      </c>
+      <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr">
         <is>
           <t>India's first 20,000mAh magnetic wireless powerbank.</t>
@@ -2496,11 +2460,7 @@
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr">
-        <is>
-          <t>6 Months (Extendable to 1 Year)</t>
-        </is>
-      </c>
+      <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
@@ -2576,7 +2536,11 @@
           <t>Pebble PB Fuel</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/rapid-fuel</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
@@ -2616,11 +2580,7 @@
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>6 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>10000 mAh total battery capacity for daily use.</t>
@@ -2636,11 +2596,7 @@
           <t>Type-C port for universal device connection.</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>6 Months Warranty coverage for product assurance.</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.pebblecart.com/products/rapid-fuel)</t>
@@ -2736,46 +2692,34 @@
       </c>
       <c r="BC12" t="inlineStr"/>
       <c r="BD12" t="inlineStr"/>
-      <c r="BE12" t="inlineStr">
+      <c r="BE12" t="inlineStr"/>
+      <c r="BF12" t="inlineStr"/>
+      <c r="BG12" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/rapid-fuel</t>
         </is>
       </c>
-      <c r="BF12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG12" t="inlineStr">
+      <c r="BH12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI12" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/rapid-fuel</t>
         </is>
       </c>
-      <c r="BH12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI12" t="inlineStr">
+      <c r="BJ12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK12" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/rapid-fuel</t>
         </is>
       </c>
-      <c r="BJ12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK12" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/rapid-fuel</t>
-        </is>
-      </c>
       <c r="BL12" t="n">
         <v>1</v>
       </c>
-      <c r="BM12" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/rapid-fuel</t>
-        </is>
-      </c>
-      <c r="BN12" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM12" t="inlineStr"/>
+      <c r="BN12" t="inlineStr"/>
       <c r="BO12" t="n">
         <v>1</v>
       </c>
@@ -2966,11 +2910,7 @@
           <t>100g</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>6 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
           <t>10000 mAh capacity stores multiple device charges safely.</t>
@@ -2986,11 +2926,7 @@
           <t>100g lightweight design ensures easy daily portability.</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>6 months warranty included against manufacturing defects.</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-rapid-air)</t>
@@ -3092,46 +3028,34 @@
       <c r="BD14" t="n">
         <v>1</v>
       </c>
-      <c r="BE14" t="inlineStr">
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
+      <c r="BG14" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
         </is>
       </c>
-      <c r="BF14" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG14" t="inlineStr">
+      <c r="BH14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI14" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
         </is>
       </c>
-      <c r="BH14" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI14" t="inlineStr">
+      <c r="BJ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK14" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
         </is>
       </c>
-      <c r="BJ14" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK14" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
-        </is>
-      </c>
       <c r="BL14" t="n">
         <v>1</v>
       </c>
-      <c r="BM14" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-rapid-air</t>
-        </is>
-      </c>
-      <c r="BN14" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
       <c r="BO14" t="n">
         <v>1</v>
       </c>
@@ -3211,11 +3135,7 @@
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>6 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>20000 mAh total power capacity for multiple device charges.</t>
@@ -3231,11 +3151,7 @@
           <t>Type-C and built-in Type-C cable ports included.</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>6 months warranty included from the date of purchase.</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.pebblecart.com/products/rapid-boost-65) + tier-1-vision: brand-page (https://www.pebblecart.com/products/rapid-boost-65)</t>
@@ -3335,46 +3251,34 @@
       </c>
       <c r="BC15" t="inlineStr"/>
       <c r="BD15" t="inlineStr"/>
-      <c r="BE15" t="inlineStr">
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/rapid-boost-65</t>
         </is>
       </c>
-      <c r="BF15" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG15" t="inlineStr">
+      <c r="BH15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI15" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/rapid-boost-65</t>
         </is>
       </c>
-      <c r="BH15" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI15" t="inlineStr">
+      <c r="BJ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK15" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/rapid-boost-65</t>
         </is>
       </c>
-      <c r="BJ15" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK15" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
-        </is>
-      </c>
       <c r="BL15" t="n">
         <v>1</v>
       </c>
-      <c r="BM15" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/rapid-boost-65</t>
-        </is>
-      </c>
-      <c r="BN15" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
       <c r="BO15" t="n">
         <v>1</v>
       </c>
@@ -3458,11 +3362,7 @@
           <t>300g</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>6 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>10000 mAh capacity stores backup power for devices.</t>
@@ -3478,11 +3378,7 @@
           <t>300g lightweight build for everyday portability.</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>6 months warranty provides standard manufacturer support.</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-rapid-electra10)</t>
@@ -3584,46 +3480,34 @@
       <c r="BD16" t="n">
         <v>1</v>
       </c>
-      <c r="BE16" t="inlineStr">
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr"/>
+      <c r="BG16" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
         </is>
       </c>
-      <c r="BF16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG16" t="inlineStr">
+      <c r="BH16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI16" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
         </is>
       </c>
-      <c r="BH16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI16" t="inlineStr">
+      <c r="BJ16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK16" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
         </is>
       </c>
-      <c r="BJ16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK16" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
-        </is>
-      </c>
       <c r="BL16" t="n">
         <v>1</v>
       </c>
-      <c r="BM16" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-rapid-electra10</t>
-        </is>
-      </c>
-      <c r="BN16" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM16" t="inlineStr"/>
+      <c r="BN16" t="inlineStr"/>
       <c r="BO16" t="n">
         <v>1</v>
       </c>
@@ -3707,11 +3591,7 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>6 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>20000 mAh capacity for multiple device charges.</t>
@@ -3727,11 +3607,7 @@
           <t>Type-C and USB-A ports for versatile connections.</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>6 months warranty coverage for reliable support.</t>
-        </is>
-      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-electra10)</t>
@@ -3833,46 +3709,34 @@
       <c r="BD17" t="n">
         <v>1</v>
       </c>
-      <c r="BE17" t="inlineStr">
+      <c r="BE17" t="inlineStr"/>
+      <c r="BF17" t="inlineStr"/>
+      <c r="BG17" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-electra10</t>
         </is>
       </c>
-      <c r="BF17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG17" t="inlineStr">
+      <c r="BH17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI17" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-electra10</t>
         </is>
       </c>
-      <c r="BH17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI17" t="inlineStr">
+      <c r="BJ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK17" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/pebble-electra10</t>
         </is>
       </c>
-      <c r="BJ17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK17" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-electra10</t>
-        </is>
-      </c>
       <c r="BL17" t="n">
         <v>1</v>
       </c>
-      <c r="BM17" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-electra10</t>
-        </is>
-      </c>
-      <c r="BN17" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM17" t="inlineStr"/>
+      <c r="BN17" t="inlineStr"/>
       <c r="BO17" t="n">
         <v>1</v>
       </c>
@@ -3956,11 +3820,7 @@
           <t>305g</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>6 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>20000 mAh capacity for extended mobile device usage.</t>
@@ -4082,14 +3942,8 @@
       <c r="BD18" t="n">
         <v>1</v>
       </c>
-      <c r="BE18" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/rapid-nova20</t>
-        </is>
-      </c>
-      <c r="BF18" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE18" t="inlineStr"/>
+      <c r="BF18" t="inlineStr"/>
       <c r="BG18" t="inlineStr">
         <is>
           <t>https://www.pebblecart.com/products/rapid-nova20</t>
@@ -4202,7 +4056,7 @@
       <c r="AK19" t="inlineStr"/>
       <c r="AL19" t="inlineStr">
         <is>
-          <t>Hard Block: All spec tiers exhausted without finding technical specifications</t>
+          <t>Skipped: Skipped: All spec tiers exhausted (including Vision) without finding technical specifications</t>
         </is>
       </c>
       <c r="AM19" t="inlineStr">
@@ -4215,7 +4069,11 @@
           <t>brand-product-page</t>
         </is>
       </c>
-      <c r="AO19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>Luxcell Mini</t>
+        </is>
+      </c>
       <c r="AP19" t="n">
         <v>2499</v>
       </c>
@@ -4251,7 +4109,8 @@
       </c>
       <c r="BQ19" t="inlineStr">
         <is>
-          <t>Attempt 1: [PB-POR-001] BLOCKED: All tiers exhausted</t>
+          <t>Attempt 1: [PB-POR-001] SKIPPED: All tiers exhausted
+Attempt 1: [PB-POR-001] SKIPPED: All tiers exhausted</t>
         </is>
       </c>
       <c r="BR19" t="inlineStr">
@@ -4288,73 +4147,21 @@
       <c r="H20" t="n">
         <v>1331</v>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Luxcell Wireless Mini</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Compact power bank featuring 10000 mAh capacity and magnetic wireless support.</t>
-        </is>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>10000 mAh</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>15W Fast Charging</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Magnetic Wireless</t>
-        </is>
-      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>10000 mAh capacity provides reliable emergency power.</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>15W fast charging delivers rapid device recovery.</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Magnetic wireless enables convenient cable-free charging.</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>12 months warranty ensures long-term dependability.</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>tier-1: brand-page (https://www.portronics.com/products/luxcell-wireless-mini-10k)</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/cdn/shop/files/Luxcell_Wireless_Mini_10K_wireless_power_bank.jpg?v=1742981494&amp;width=2048</t>
-        </is>
-      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr">
         <is>
           <t>ok</t>
@@ -4375,12 +4182,12 @@
       <c r="AK20" t="inlineStr"/>
       <c r="AL20" t="inlineStr">
         <is>
-          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
+          <t>Skipped: Skipped: All spec tiers exhausted (including Vision) without finding technical specifications</t>
         </is>
       </c>
       <c r="AM20" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="AN20" t="inlineStr">
@@ -4390,96 +4197,36 @@
       </c>
       <c r="AO20" t="inlineStr">
         <is>
-          <t>Wireless Mini</t>
+          <t>Luxcell</t>
         </is>
       </c>
       <c r="AP20" t="n">
         <v>3999</v>
       </c>
-      <c r="AQ20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="AR20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="AT20" t="n">
-        <v>1</v>
-      </c>
+      <c r="AQ20" t="inlineStr"/>
+      <c r="AR20" t="inlineStr"/>
+      <c r="AS20" t="inlineStr"/>
+      <c r="AT20" t="inlineStr"/>
       <c r="AU20" t="inlineStr"/>
       <c r="AV20" t="inlineStr"/>
-      <c r="AW20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="AX20" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="AZ20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BA20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="BB20" t="n">
-        <v>1</v>
-      </c>
+      <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+      <c r="AZ20" t="inlineStr"/>
+      <c r="BA20" t="inlineStr"/>
+      <c r="BB20" t="inlineStr"/>
       <c r="BC20" t="inlineStr"/>
       <c r="BD20" t="inlineStr"/>
-      <c r="BE20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="BF20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="BH20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="BJ20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="BL20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM20" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-wireless-mini-10k</t>
-        </is>
-      </c>
-      <c r="BN20" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE20" t="inlineStr"/>
+      <c r="BF20" t="inlineStr"/>
+      <c r="BG20" t="inlineStr"/>
+      <c r="BH20" t="inlineStr"/>
+      <c r="BI20" t="inlineStr"/>
+      <c r="BJ20" t="inlineStr"/>
+      <c r="BK20" t="inlineStr"/>
+      <c r="BL20" t="inlineStr"/>
+      <c r="BM20" t="inlineStr"/>
+      <c r="BN20" t="inlineStr"/>
       <c r="BO20" t="n">
         <v>1</v>
       </c>
@@ -4488,7 +4235,8 @@
       </c>
       <c r="BQ20" t="inlineStr">
         <is>
-          <t>Attempt 1: [PB-POR-002] Collected via tier-1: brand-page (https://www.portronics.com/products/luxcell-wireless-mini-10k)</t>
+          <t>Attempt 1: [PB-POR-002] Collected via tier-1: brand-page (https://www.portronics.com/products/luxcell-wireless-mini-10k)
+Attempt 1: [PB-POR-002] SKIPPED: All tiers exhausted</t>
         </is>
       </c>
       <c r="BR20" t="inlineStr">
@@ -4557,11 +4305,7 @@
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>10000 mAh capacity stores backup power for devices.</t>
@@ -4577,11 +4321,7 @@
           <t>Type-C input allows standard cable connection.</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>12 Months Warranty provides official service cover.</t>
-        </is>
-      </c>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.portronics.com/products/luxcell-b12-type-c-input)</t>
@@ -4677,46 +4417,34 @@
       </c>
       <c r="BC21" t="inlineStr"/>
       <c r="BD21" t="inlineStr"/>
-      <c r="BE21" t="inlineStr">
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
         </is>
       </c>
-      <c r="BF21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG21" t="inlineStr">
+      <c r="BH21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI21" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
         </is>
       </c>
-      <c r="BH21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI21" t="inlineStr">
+      <c r="BJ21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK21" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
         </is>
       </c>
-      <c r="BJ21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK21" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
-        </is>
-      </c>
       <c r="BL21" t="n">
         <v>1</v>
       </c>
-      <c r="BM21" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-b12-type-c-input</t>
-        </is>
-      </c>
-      <c r="BN21" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
       <c r="BO21" t="n">
         <v>1</v>
       </c>
@@ -4794,11 +4522,7 @@
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
           <t>10000 mAh capacity provides reliable backup power.</t>
@@ -4814,11 +4538,7 @@
           <t>Type-C and magnetic wireless ports offer charging.</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>12 months warranty ensures long-term product trust.</t>
-        </is>
-      </c>
+      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.portronics.com/products/power-shutter)</t>
@@ -4914,46 +4634,34 @@
       </c>
       <c r="BC22" t="inlineStr"/>
       <c r="BD22" t="inlineStr"/>
-      <c r="BE22" t="inlineStr">
+      <c r="BE22" t="inlineStr"/>
+      <c r="BF22" t="inlineStr"/>
+      <c r="BG22" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/power-shutter</t>
         </is>
       </c>
-      <c r="BF22" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG22" t="inlineStr">
+      <c r="BH22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI22" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/power-shutter</t>
         </is>
       </c>
-      <c r="BH22" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI22" t="inlineStr">
+      <c r="BJ22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK22" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/power-shutter</t>
         </is>
       </c>
-      <c r="BJ22" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK22" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/power-shutter</t>
-        </is>
-      </c>
       <c r="BL22" t="n">
         <v>1</v>
       </c>
-      <c r="BM22" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/power-shutter</t>
-        </is>
-      </c>
-      <c r="BN22" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM22" t="inlineStr"/>
+      <c r="BN22" t="inlineStr"/>
       <c r="BO22" t="n">
         <v>1</v>
       </c>
@@ -5027,11 +4735,7 @@
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>10000 mAh capacity supports daily power needs.</t>
@@ -5044,14 +4748,10 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>12 months warranty provides manufacturer support.</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
           <t>Compact design ensures easy everyday carry.</t>
         </is>
       </c>
+      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
           <t>tier-2: brand-collection (https://www.portronics.com/products/power-shutter-pro)</t>
@@ -5141,14 +4841,8 @@
       <c r="BB23" t="inlineStr"/>
       <c r="BC23" t="inlineStr"/>
       <c r="BD23" t="inlineStr"/>
-      <c r="BE23" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/power-shutter-pro</t>
-        </is>
-      </c>
-      <c r="BF23" t="n">
-        <v>2</v>
-      </c>
+      <c r="BE23" t="inlineStr"/>
+      <c r="BF23" t="inlineStr"/>
       <c r="BG23" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/power-shutter-pro</t>
@@ -5173,14 +4867,8 @@
       <c r="BL23" t="n">
         <v>2</v>
       </c>
-      <c r="BM23" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/power-shutter-pro</t>
-        </is>
-      </c>
-      <c r="BN23" t="n">
-        <v>2</v>
-      </c>
+      <c r="BM23" t="inlineStr"/>
+      <c r="BN23" t="inlineStr"/>
       <c r="BO23" t="n">
         <v>1</v>
       </c>
@@ -5258,11 +4946,7 @@
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>10000 mAh capacity for multiple device charges.</t>
@@ -5278,11 +4962,7 @@
           <t>Type-C and magnetic wireless ports included.</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>12 months warranty coverage for peace of mind.</t>
-        </is>
-      </c>
+      <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.portronics.com/products/chyro)</t>
@@ -5378,46 +5058,34 @@
       </c>
       <c r="BC24" t="inlineStr"/>
       <c r="BD24" t="inlineStr"/>
-      <c r="BE24" t="inlineStr">
+      <c r="BE24" t="inlineStr"/>
+      <c r="BF24" t="inlineStr"/>
+      <c r="BG24" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/chyro</t>
         </is>
       </c>
-      <c r="BF24" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG24" t="inlineStr">
+      <c r="BH24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI24" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/chyro</t>
         </is>
       </c>
-      <c r="BH24" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI24" t="inlineStr">
+      <c r="BJ24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK24" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/chyro</t>
         </is>
       </c>
-      <c r="BJ24" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK24" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/chyro</t>
-        </is>
-      </c>
       <c r="BL24" t="n">
         <v>1</v>
       </c>
-      <c r="BM24" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/chyro</t>
-        </is>
-      </c>
-      <c r="BN24" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM24" t="inlineStr"/>
+      <c r="BN24" t="inlineStr"/>
       <c r="BO24" t="n">
         <v>1</v>
       </c>
@@ -5495,11 +5163,7 @@
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
           <t>20000 mAh capacity provides multiple device charges.</t>
@@ -5515,11 +5179,7 @@
           <t>Type-C and magnetic wireless ports offer versatile use.</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>12 months warranty ensures reliable long-term support.</t>
-        </is>
-      </c>
+      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.portronics.com/products/power-shutter-air-20k)</t>
@@ -5615,46 +5275,34 @@
       </c>
       <c r="BC25" t="inlineStr"/>
       <c r="BD25" t="inlineStr"/>
-      <c r="BE25" t="inlineStr">
+      <c r="BE25" t="inlineStr"/>
+      <c r="BF25" t="inlineStr"/>
+      <c r="BG25" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/power-shutter-air-20k</t>
         </is>
       </c>
-      <c r="BF25" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG25" t="inlineStr">
+      <c r="BH25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI25" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/power-shutter-air-20k</t>
         </is>
       </c>
-      <c r="BH25" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI25" t="inlineStr">
+      <c r="BJ25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK25" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/power-shutter-air-20k</t>
         </is>
       </c>
-      <c r="BJ25" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK25" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
-        </is>
-      </c>
       <c r="BL25" t="n">
         <v>1</v>
       </c>
-      <c r="BM25" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/power-shutter-air-20k</t>
-        </is>
-      </c>
-      <c r="BN25" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM25" t="inlineStr"/>
+      <c r="BN25" t="inlineStr"/>
       <c r="BO25" t="n">
         <v>1</v>
       </c>
@@ -5731,7 +5379,7 @@
       <c r="AK26" t="inlineStr"/>
       <c r="AL26" t="inlineStr">
         <is>
-          <t>Hard Block: All spec tiers exhausted without finding technical specifications</t>
+          <t>Skipped: Skipped: All spec tiers exhausted (including Vision) without finding technical specifications</t>
         </is>
       </c>
       <c r="AM26" t="inlineStr">
@@ -5774,7 +5422,12 @@
       </c>
       <c r="BQ26" t="inlineStr">
         <is>
-          <t>Attempt 1: [PB-POR-008] BLOCKED: All tiers exhausted</t>
+          <t>Attempt 1: [PB-POR-008] BLOCKED: All tiers exhausted
+Attempt 1: [PB-POR-008] SKIPPED: All tiers exhausted
+Cleaned Display_Name to 'nan'
+Attempt 1: [PB-POR-008] SKIPPED: All tiers exhausted
+Cleaned Display_Name to 'nan'
+Cleaned Display_Name to 'nan'</t>
         </is>
       </c>
       <c r="BR26" t="inlineStr"/>
@@ -5839,11 +5492,7 @@
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>10000 mAh total capacity for multiple device charges.</t>
@@ -5859,11 +5508,7 @@
           <t>Type-C and USB-A ports for versatile connectivity.</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>12 Months Warranty included for product assurance.</t>
-        </is>
-      </c>
+      <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.portronics.com/products/luxcell-uno-10)</t>
@@ -5959,46 +5604,34 @@
       </c>
       <c r="BC27" t="inlineStr"/>
       <c r="BD27" t="inlineStr"/>
-      <c r="BE27" t="inlineStr">
+      <c r="BE27" t="inlineStr"/>
+      <c r="BF27" t="inlineStr"/>
+      <c r="BG27" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/luxcell-uno-10</t>
         </is>
       </c>
-      <c r="BF27" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG27" t="inlineStr">
+      <c r="BH27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI27" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/luxcell-uno-10</t>
         </is>
       </c>
-      <c r="BH27" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI27" t="inlineStr">
+      <c r="BJ27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK27" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/luxcell-uno-10</t>
         </is>
       </c>
-      <c r="BJ27" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK27" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-uno-10</t>
-        </is>
-      </c>
       <c r="BL27" t="n">
         <v>1</v>
       </c>
-      <c r="BM27" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/luxcell-uno-10</t>
-        </is>
-      </c>
-      <c r="BN27" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM27" t="inlineStr"/>
+      <c r="BN27" t="inlineStr"/>
       <c r="BO27" t="n">
         <v>1</v>
       </c>
@@ -6076,11 +5709,7 @@
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
           <t>10000 mAh capacity for extended mobile device usage.</t>
@@ -6096,11 +5725,7 @@
           <t>Type-C and magnetic wireless ports for dual charging.</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>12 months warranty included for long-term reliability.</t>
-        </is>
-      </c>
+      <c r="U28" t="inlineStr"/>
       <c r="V28" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.portronics.com/products/revvo)</t>
@@ -6196,46 +5821,34 @@
       </c>
       <c r="BC28" t="inlineStr"/>
       <c r="BD28" t="inlineStr"/>
-      <c r="BE28" t="inlineStr">
+      <c r="BE28" t="inlineStr"/>
+      <c r="BF28" t="inlineStr"/>
+      <c r="BG28" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/revvo</t>
         </is>
       </c>
-      <c r="BF28" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG28" t="inlineStr">
+      <c r="BH28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI28" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/revvo</t>
         </is>
       </c>
-      <c r="BH28" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI28" t="inlineStr">
+      <c r="BJ28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK28" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/revvo</t>
         </is>
       </c>
-      <c r="BJ28" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK28" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/revvo</t>
-        </is>
-      </c>
       <c r="BL28" t="n">
         <v>1</v>
       </c>
-      <c r="BM28" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/revvo</t>
-        </is>
-      </c>
-      <c r="BN28" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM28" t="inlineStr"/>
+      <c r="BN28" t="inlineStr"/>
       <c r="BO28" t="n">
         <v>1</v>
       </c>
@@ -6366,7 +5979,10 @@
       <c r="BQ29" t="inlineStr">
         <is>
           <t>Attempt 1: [PB-POR-011] Collected via tier-1: brand-page (https://www.portronics.com/products/power-shutter)
-Attempt 1: No automated fix available for flags: ['Duplicate image asset: identical file hash to product [PB-POR-004]']</t>
+Attempt 1: No automated fix available for flags: ['Duplicate image asset: identical file hash to product [PB-POR-004]']
+Cleaned Display_Name to 'nan'
+Cleaned Display_Name to 'nan'
+Cleaned Display_Name to 'nan'</t>
         </is>
       </c>
       <c r="BR29" t="inlineStr">
@@ -6477,7 +6093,10 @@
       </c>
       <c r="BQ30" t="inlineStr">
         <is>
-          <t>Attempt 1: [PB-POR-012] BLOCKED: All tiers exhausted</t>
+          <t>Attempt 1: [PB-POR-012] BLOCKED: All tiers exhausted
+Cleaned Display_Name to 'nan'
+Cleaned Display_Name to 'nan'
+Cleaned Display_Name to 'nan'</t>
         </is>
       </c>
       <c r="BR30" t="inlineStr"/>
@@ -6542,11 +6161,7 @@
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>12 Months Warranty</t>
-        </is>
-      </c>
+      <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
           <t>20000 mAh capacity provides multiple device charges.</t>
@@ -6562,11 +6177,7 @@
           <t>Type-C and USB-A ports enable dual device charging.</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>12 months warranty ensures long term reliability.</t>
-        </is>
-      </c>
+      <c r="U31" t="inlineStr"/>
       <c r="V31" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.portronics.com/products/aero-65)</t>
@@ -6662,46 +6273,34 @@
       </c>
       <c r="BC31" t="inlineStr"/>
       <c r="BD31" t="inlineStr"/>
-      <c r="BE31" t="inlineStr">
+      <c r="BE31" t="inlineStr"/>
+      <c r="BF31" t="inlineStr"/>
+      <c r="BG31" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/aero-65</t>
         </is>
       </c>
-      <c r="BF31" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG31" t="inlineStr">
+      <c r="BH31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI31" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/aero-65</t>
         </is>
       </c>
-      <c r="BH31" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI31" t="inlineStr">
+      <c r="BJ31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK31" t="inlineStr">
         <is>
           <t>https://www.portronics.com/products/aero-65</t>
         </is>
       </c>
-      <c r="BJ31" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK31" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/aero-65</t>
-        </is>
-      </c>
       <c r="BL31" t="n">
         <v>1</v>
       </c>
-      <c r="BM31" t="inlineStr">
-        <is>
-          <t>https://www.portronics.com/products/aero-65</t>
-        </is>
-      </c>
-      <c r="BN31" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM31" t="inlineStr"/>
+      <c r="BN31" t="inlineStr"/>
       <c r="BO31" t="n">
         <v>1</v>
       </c>
@@ -6779,11 +6378,7 @@
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>10000 mAh capacity provides reliable mobile device power.</t>
@@ -6799,11 +6394,7 @@
           <t>1 type-c port handles both device charge and recharge.</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>1 year warranty is included for product protection.</t>
-        </is>
-      </c>
+      <c r="U32" t="inlineStr"/>
       <c r="V32" t="inlineStr">
         <is>
           <t>tier-0-vision: (brochure: urbn_catalog.pdf, page 3)</t>
@@ -6903,56 +6494,40 @@
       </c>
       <c r="BC32" t="inlineStr"/>
       <c r="BD32" t="inlineStr"/>
-      <c r="BE32" t="inlineStr">
+      <c r="BE32" t="inlineStr"/>
+      <c r="BF32" t="inlineStr"/>
+      <c r="BG32" t="inlineStr">
         <is>
           <t>brochure: urbn_catalog.pdf, page 3</t>
         </is>
       </c>
-      <c r="BF32" t="inlineStr">
+      <c r="BH32" t="inlineStr">
         <is>
           <t>0-vision</t>
         </is>
       </c>
-      <c r="BG32" t="inlineStr">
+      <c r="BI32" t="inlineStr">
         <is>
           <t>brochure: urbn_catalog.pdf, page 3</t>
         </is>
       </c>
-      <c r="BH32" t="inlineStr">
+      <c r="BJ32" t="inlineStr">
         <is>
           <t>0-vision</t>
         </is>
       </c>
-      <c r="BI32" t="inlineStr">
+      <c r="BK32" t="inlineStr">
         <is>
           <t>brochure: urbn_catalog.pdf, page 3</t>
         </is>
       </c>
-      <c r="BJ32" t="inlineStr">
+      <c r="BL32" t="inlineStr">
         <is>
           <t>0-vision</t>
         </is>
       </c>
-      <c r="BK32" t="inlineStr">
-        <is>
-          <t>brochure: urbn_catalog.pdf, page 3</t>
-        </is>
-      </c>
-      <c r="BL32" t="inlineStr">
-        <is>
-          <t>0-vision</t>
-        </is>
-      </c>
-      <c r="BM32" t="inlineStr">
-        <is>
-          <t>brochure: urbn_catalog.pdf, page 3</t>
-        </is>
-      </c>
-      <c r="BN32" t="inlineStr">
-        <is>
-          <t>0-vision</t>
-        </is>
-      </c>
+      <c r="BM32" t="inlineStr"/>
+      <c r="BN32" t="inlineStr"/>
       <c r="BO32" t="n">
         <v>1</v>
       </c>
@@ -7036,11 +6611,7 @@
           <t>205g</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
           <t>10000 mAh capacity provides reliable mobile power.</t>
@@ -7166,14 +6737,8 @@
       <c r="BD33" t="n">
         <v>1</v>
       </c>
-      <c r="BE33" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF33" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE33" t="inlineStr"/>
+      <c r="BF33" t="inlineStr"/>
       <c r="BG33" t="inlineStr">
         <is>
           <t>https://www.urbnworld.com/products/10-000-mah-atom-link</t>
@@ -7283,11 +6848,7 @@
         </is>
       </c>
       <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
           <t>10000mAh capacity provides reliable backup power.</t>
@@ -7398,14 +6959,8 @@
       </c>
       <c r="BC34" t="inlineStr"/>
       <c r="BD34" t="inlineStr"/>
-      <c r="BE34" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF34" t="n">
-        <v>0</v>
-      </c>
+      <c r="BE34" t="inlineStr"/>
+      <c r="BF34" t="inlineStr"/>
       <c r="BG34" t="inlineStr">
         <is>
           <t>brochure: urbn_catalog.pdf, page 13</t>
@@ -7521,11 +7076,7 @@
           <t>234g</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
           <t>10000 mAh capacity provides multiple device charges.</t>
@@ -7651,14 +7202,8 @@
       <c r="BD35" t="n">
         <v>1</v>
       </c>
-      <c r="BE35" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF35" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE35" t="inlineStr"/>
+      <c r="BF35" t="inlineStr"/>
       <c r="BG35" t="inlineStr">
         <is>
           <t>https://www.urbnworld.com/products/10-000mah-flux-qi2-magtag-power-bank</t>
@@ -7883,11 +7428,7 @@
           <t>195g</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
           <t>10000 mAh total capacity for daily device charging needs.</t>
@@ -8009,14 +7550,8 @@
       <c r="BD37" t="n">
         <v>1</v>
       </c>
-      <c r="BE37" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF37" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE37" t="inlineStr"/>
+      <c r="BF37" t="inlineStr"/>
       <c r="BG37" t="inlineStr">
         <is>
           <t>https://www.urbnworld.com/products/10000mah-curve-magatg-power-bank</t>
@@ -8132,11 +7667,7 @@
           <t>220g</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
           <t>10000 mAh capacity with built-in Li-Polymer battery cells.</t>
@@ -8152,11 +7683,7 @@
           <t>12 layers of protection ensuring safe daily device usage.</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>6 months manufacturer warranty included with purchase.</t>
-        </is>
-      </c>
+      <c r="U38" t="inlineStr"/>
       <c r="V38" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank) + tier-3: retail-reliance (https://www.reliancedigital.in/product/urbn-10000-mah-15-w-arc-magtag-power-bank-with-stand-black-mgp5oz-9546389)</t>
@@ -8258,14 +7785,8 @@
       <c r="BD38" t="n">
         <v>3</v>
       </c>
-      <c r="BE38" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF38" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE38" t="inlineStr"/>
+      <c r="BF38" t="inlineStr"/>
       <c r="BG38" t="inlineStr">
         <is>
           <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
@@ -8290,14 +7811,8 @@
       <c r="BL38" t="n">
         <v>1</v>
       </c>
-      <c r="BM38" t="inlineStr">
-        <is>
-          <t>https://www.urbnworld.com/products/urbn-10000-mah-arc-magtag-power-bank</t>
-        </is>
-      </c>
-      <c r="BN38" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM38" t="inlineStr"/>
+      <c r="BN38" t="inlineStr"/>
       <c r="BO38" t="n">
         <v>1</v>
       </c>
@@ -8381,11 +7896,7 @@
           <t>180g</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
           <t>10000 mAh capacity stores multiple full charges.</t>
@@ -8511,14 +8022,8 @@
       <c r="BD39" t="n">
         <v>1</v>
       </c>
-      <c r="BE39" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF39" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE39" t="inlineStr"/>
+      <c r="BF39" t="inlineStr"/>
       <c r="BG39" t="inlineStr">
         <is>
           <t>https://www.urbnworld.com/products/10-000mah-mini-volt-35w-power-bank</t>
@@ -8634,11 +8139,7 @@
           <t>194g</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
           <t>10000mAh capacity provides multiple full device charges.</t>
@@ -8764,14 +8265,8 @@
       <c r="BD40" t="n">
         <v>1</v>
       </c>
-      <c r="BE40" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF40" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE40" t="inlineStr"/>
+      <c r="BF40" t="inlineStr"/>
       <c r="BG40" t="inlineStr">
         <is>
           <t>https://www.urbnworld.com/products/10-000-mah-aero-magtag-power-bank</t>
@@ -8887,11 +8382,7 @@
           <t>200g</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>10000 mAh capacity provides reliable mobile backup power.</t>
@@ -9017,14 +8508,8 @@
       <c r="BD41" t="n">
         <v>1</v>
       </c>
-      <c r="BE41" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF41" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE41" t="inlineStr"/>
+      <c r="BF41" t="inlineStr"/>
       <c r="BG41" t="inlineStr">
         <is>
           <t>https://www.urbnworld.com/products/10-000mah-slate-qi2-magtag-power-bank</t>
@@ -9140,11 +8625,7 @@
           <t>343g</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>1 Year</t>
-        </is>
-      </c>
+      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>20000 mAh capacity stores multiple full device charges.</t>
@@ -9270,14 +8751,8 @@
       <c r="BD42" t="n">
         <v>1</v>
       </c>
-      <c r="BE42" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF42" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE42" t="inlineStr"/>
+      <c r="BF42" t="inlineStr"/>
       <c r="BG42" t="inlineStr">
         <is>
           <t>https://www.urbnworld.com/products/20-000mah-ultra-volt-65w</t>
@@ -9391,11 +8866,7 @@
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>2 Years</t>
-        </is>
-      </c>
+      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>10000mAh capacity provides reliable backup power.</t>
@@ -9411,11 +8882,7 @@
           <t>Type-C and Micro-USB ports offer dual input.</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>2 years manufacture warranty included for users.</t>
-        </is>
-      </c>
+      <c r="U43" t="inlineStr"/>
       <c r="V43" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://evmzone.com/evm-products/encharge.html)</t>
@@ -9511,14 +8978,8 @@
       </c>
       <c r="BC43" t="inlineStr"/>
       <c r="BD43" t="inlineStr"/>
-      <c r="BE43" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF43" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE43" t="inlineStr"/>
+      <c r="BF43" t="inlineStr"/>
       <c r="BG43" t="inlineStr">
         <is>
           <t>https://evmzone.com/evm-products/encharge.html</t>
@@ -9543,14 +9004,8 @@
       <c r="BL43" t="n">
         <v>1</v>
       </c>
-      <c r="BM43" t="inlineStr">
-        <is>
-          <t>https://evmzone.com/evm-products/encharge.html</t>
-        </is>
-      </c>
-      <c r="BN43" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM43" t="inlineStr"/>
+      <c r="BN43" t="inlineStr"/>
       <c r="BO43" t="n">
         <v>1</v>
       </c>
@@ -9634,11 +9089,7 @@
         </is>
       </c>
       <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>2 Years</t>
-        </is>
-      </c>
+      <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
           <t>10000 mAh capacity for multiple device charges.</t>
@@ -9756,14 +9207,8 @@
       </c>
       <c r="BC44" t="inlineStr"/>
       <c r="BD44" t="inlineStr"/>
-      <c r="BE44" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF44" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE44" t="inlineStr"/>
+      <c r="BF44" t="inlineStr"/>
       <c r="BG44" t="inlineStr">
         <is>
           <t>https://evmzone.com/evm-products/powerbank/enbolt-power-bank-10000mah.html</t>
@@ -9877,11 +9322,7 @@
         </is>
       </c>
       <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>2 Years</t>
-        </is>
-      </c>
+      <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
           <t>10000 mAh capacity supports extended power needs.</t>
@@ -9997,14 +9438,8 @@
       </c>
       <c r="BC45" t="inlineStr"/>
       <c r="BD45" t="inlineStr"/>
-      <c r="BE45" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF45" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE45" t="inlineStr"/>
+      <c r="BF45" t="inlineStr"/>
       <c r="BG45" t="inlineStr">
         <is>
           <t>https://evmzone.com/enmag-ace-power-bank-evm-p0301.html</t>
@@ -10120,11 +9555,7 @@
         </is>
       </c>
       <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>2 Years Warranty</t>
-        </is>
-      </c>
+      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>10000mAh capacity provides backup power for mobile devices.</t>
@@ -10140,11 +9571,7 @@
           <t>2.4 Amp output delivers fast charging capabilities.</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>2 years warranty included from the date of purchase.</t>
-        </is>
-      </c>
+      <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
           <t>tier-1: brand-page (https://evmzone.com/evm-products/powerbank/encase-power-bank.html)</t>
@@ -10240,46 +9667,34 @@
       </c>
       <c r="BC46" t="inlineStr"/>
       <c r="BD46" t="inlineStr"/>
-      <c r="BE46" t="inlineStr">
+      <c r="BE46" t="inlineStr"/>
+      <c r="BF46" t="inlineStr"/>
+      <c r="BG46" t="inlineStr">
         <is>
           <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
         </is>
       </c>
-      <c r="BF46" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG46" t="inlineStr">
+      <c r="BH46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI46" t="inlineStr">
         <is>
           <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
         </is>
       </c>
-      <c r="BH46" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI46" t="inlineStr">
+      <c r="BJ46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK46" t="inlineStr">
         <is>
           <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
         </is>
       </c>
-      <c r="BJ46" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK46" t="inlineStr">
-        <is>
-          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
-        </is>
-      </c>
       <c r="BL46" t="n">
         <v>1</v>
       </c>
-      <c r="BM46" t="inlineStr">
-        <is>
-          <t>https://evmzone.com/evm-products/powerbank/encase-power-bank.html</t>
-        </is>
-      </c>
-      <c r="BN46" t="n">
-        <v>1</v>
-      </c>
+      <c r="BM46" t="inlineStr"/>
+      <c r="BN46" t="inlineStr"/>
       <c r="BO46" t="n">
         <v>1</v>
       </c>
@@ -10362,11 +9777,7 @@
         </is>
       </c>
       <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>2 Years</t>
-        </is>
-      </c>
+      <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
           <t>10000mAh Li-polymer battery capacity for daily use.</t>
@@ -10482,14 +9893,8 @@
       </c>
       <c r="BC47" t="inlineStr"/>
       <c r="BD47" t="inlineStr"/>
-      <c r="BE47" t="inlineStr">
-        <is>
-          <t>brand-default-policy</t>
-        </is>
-      </c>
-      <c r="BF47" t="n">
-        <v>1</v>
-      </c>
+      <c r="BE47" t="inlineStr"/>
+      <c r="BF47" t="inlineStr"/>
       <c r="BG47" t="inlineStr">
         <is>
           <t>https://evmzone.com/evm-products/powerbank/enmove.html</t>
@@ -10540,6 +9945,484 @@
         </is>
       </c>
       <c r="BS47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PB-GG-001</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Powerbank</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Glow Gadget</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Ray</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/collections/powerbanks</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>1077</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Glow Ray 10000mAh</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Compact power bank featuring 10000 mAh capacity and magnetic wireless output.</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>15W Fast Charging</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Magnetic Wireless</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity for extended mobile device power.</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>15W fast charging output for rapid device charging.</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Magnetic wireless ports for cable-free convenience.</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>345g total weight designed for portable daily carry.</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2)</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/cdn/shop/files/Ray.jpg?v=1742555497&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr"/>
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr"/>
+      <c r="AD48" t="inlineStr"/>
+      <c r="AE48" t="inlineStr"/>
+      <c r="AF48" t="inlineStr"/>
+      <c r="AG48" t="inlineStr"/>
+      <c r="AH48" t="inlineStr"/>
+      <c r="AI48" t="inlineStr"/>
+      <c r="AJ48" t="inlineStr"/>
+      <c r="AK48" t="inlineStr"/>
+      <c r="AL48" t="inlineStr">
+        <is>
+          <t>URL slug numeric token mismatch: slug 'ray-customized-suction-with-wireless-fast-charging-2' contains numbers ['2'] but title/model contains ['10000'] (potential reused URL handle)</t>
+        </is>
+      </c>
+      <c r="AM48" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AN48" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AO48" t="inlineStr">
+        <is>
+          <t>Ray</t>
+        </is>
+      </c>
+      <c r="AP48" t="n">
+        <v>4199</v>
+      </c>
+      <c r="AQ48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="AR48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="AT48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU48" t="inlineStr"/>
+      <c r="AV48" t="inlineStr"/>
+      <c r="AW48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="AX48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="AZ48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="BB48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="BD48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE48" t="inlineStr"/>
+      <c r="BF48" t="inlineStr"/>
+      <c r="BG48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="BH48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="BJ48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="BL48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM48" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2</t>
+        </is>
+      </c>
+      <c r="BN48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP48" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ48" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-GG-001] Collected via tier-1: brand-page (https://glowgadgets.in/products/ray-customized-suction-with-wireless-fast-charging-2)</t>
+        </is>
+      </c>
+      <c r="BR48" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PB-GG-002</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Powerbank</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Glow Gadget</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Beam</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/collections/powerbanks</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>925</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Beam Power Bank</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Reliable 10000mAh capacity for charging devices on the go.</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>10000 mAh</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>5W Fast Charging</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, Micro-USB, Magnetic Wireless, Lightning</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>325g</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>10000 mAh capacity ensures reliable power for devices.</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>5W wireless charging supports compatible devices.</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>325g weight makes it compact and easy to carry.</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Type-C, USB-A, and Micro-USB ports provide versatility.</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://glowgadgets.in/products/beam-customized-wireless-powerbank)</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/cdn/shop/files/Beam.jpg?v=1742976064&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr"/>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
+      <c r="AD49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr"/>
+      <c r="AF49" t="inlineStr"/>
+      <c r="AG49" t="inlineStr"/>
+      <c r="AH49" t="inlineStr"/>
+      <c r="AI49" t="inlineStr"/>
+      <c r="AJ49" t="inlineStr"/>
+      <c r="AK49" t="inlineStr"/>
+      <c r="AL49" t="inlineStr"/>
+      <c r="AM49" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AN49" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AO49" t="inlineStr">
+        <is>
+          <t>Beam</t>
+        </is>
+      </c>
+      <c r="AP49" t="n">
+        <v>3999</v>
+      </c>
+      <c r="AQ49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="AR49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="AT49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU49" t="inlineStr"/>
+      <c r="AV49" t="inlineStr"/>
+      <c r="AW49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="AX49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="AZ49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="BB49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="BD49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE49" t="inlineStr"/>
+      <c r="BF49" t="inlineStr"/>
+      <c r="BG49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="BH49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="BJ49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="BL49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM49" t="inlineStr">
+        <is>
+          <t>https://glowgadgets.in/products/beam-customized-wireless-powerbank</t>
+        </is>
+      </c>
+      <c r="BN49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP49" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ49" t="inlineStr">
+        <is>
+          <t>Attempt 1: [PB-GG-002] Collected via tier-1: brand-page (https://glowgadgets.in/products/beam-customized-wireless-powerbank)</t>
+        </is>
+      </c>
+      <c r="BR49" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: purge TWS test data for clean re-test
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -2796,7 +2796,7 @@
       <c r="AK13" t="inlineStr"/>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>Hard Block: All spec tiers exhausted without finding technical specifications</t>
+          <t>Skipped: Skipped: All spec tiers exhausted (including Vision) without finding technical specifications</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
@@ -2837,9 +2837,7 @@
       </c>
       <c r="BQ13" t="inlineStr">
         <is>
-          <t>Attempt 1: [PB-PEB-002] BLOCKED: All tiers exhausted
-Cleaned Display_Name to 'nan'
-Cleaned Display_Name to 'nan'</t>
+          <t>Attempt 1: [PB-PEB-002] SKIPPED: All tiers exhausted</t>
         </is>
       </c>
       <c r="BR13" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: preserve functional model names in Ingest and add category-derived descriptor scoping with token-boundary equivalence
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS49"/>
+  <dimension ref="A1:BS52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10422,6 +10422,639 @@
       </c>
       <c r="BS49" t="inlineStr"/>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TWS-PEB-001</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Open Loop</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/open-loop</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Open Loop TWS</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Equipped with environmental noise cancellation for clear audio performance.</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Environmental Noise Cancellation</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Features advanced environmental noise cancellation.</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Designed for reliable everyday audio usage.</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/open-loop)</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/0_4af773c0-f1d6-4aa9-8aee-9095c75da084.jpg?v=1779955140&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr"/>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr"/>
+      <c r="AI50" t="inlineStr"/>
+      <c r="AJ50" t="inlineStr"/>
+      <c r="AK50" t="inlineStr"/>
+      <c r="AL50" t="inlineStr"/>
+      <c r="AM50" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AN50" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AO50" t="inlineStr">
+        <is>
+          <t>Open Loop</t>
+        </is>
+      </c>
+      <c r="AP50" t="n">
+        <v>4999</v>
+      </c>
+      <c r="AQ50" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/open-loop</t>
+        </is>
+      </c>
+      <c r="AR50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS50" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/open-loop</t>
+        </is>
+      </c>
+      <c r="AT50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU50" t="inlineStr"/>
+      <c r="AV50" t="inlineStr"/>
+      <c r="AW50" t="inlineStr"/>
+      <c r="AX50" t="inlineStr"/>
+      <c r="AY50" t="inlineStr"/>
+      <c r="AZ50" t="inlineStr"/>
+      <c r="BA50" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/open-loop</t>
+        </is>
+      </c>
+      <c r="BB50" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC50" t="inlineStr"/>
+      <c r="BD50" t="inlineStr"/>
+      <c r="BE50" t="inlineStr"/>
+      <c r="BF50" t="inlineStr"/>
+      <c r="BG50" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/open-loop</t>
+        </is>
+      </c>
+      <c r="BH50" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI50" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/open-loop</t>
+        </is>
+      </c>
+      <c r="BJ50" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK50" t="inlineStr"/>
+      <c r="BL50" t="inlineStr"/>
+      <c r="BM50" t="inlineStr"/>
+      <c r="BN50" t="inlineStr"/>
+      <c r="BO50" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP50" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ50" t="inlineStr">
+        <is>
+          <t>Attempt 1: [TWS-PEB-001] Collected via tier-1: brand-page (https://www.pebblecart.com/products/open-loop)</t>
+        </is>
+      </c>
+      <c r="BR50" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TWS-PEB-002</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>STRIKER Buds</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>STRIKER Buds</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Equipped with advanced bluetooth connectivity and quad mic environmental noise.</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>13mm Drivers</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Quad Mic ENC</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Bluetooth v5.4</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>13mm drivers deliver high quality audio output.</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Bluetooth v5.4 provides stable wireless connection.</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Quad mic ENC ensures clear call performance.</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Type-C charging port enables fast power replenishment.</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/striker-buds-tws)</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/0_e60ef5ad-0831-4ed7-ab69-28c47ef8c9fc.jpg?v=1759139099&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr"/>
+      <c r="AF51" t="inlineStr"/>
+      <c r="AG51" t="inlineStr"/>
+      <c r="AH51" t="inlineStr"/>
+      <c r="AI51" t="inlineStr"/>
+      <c r="AJ51" t="inlineStr"/>
+      <c r="AK51" t="inlineStr"/>
+      <c r="AL51" t="inlineStr"/>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AN51" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AO51" t="inlineStr">
+        <is>
+          <t>STRIKER</t>
+        </is>
+      </c>
+      <c r="AP51" t="n">
+        <v>3499</v>
+      </c>
+      <c r="AQ51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="AR51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="AT51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU51" t="inlineStr"/>
+      <c r="AV51" t="inlineStr"/>
+      <c r="AW51" t="inlineStr"/>
+      <c r="AX51" t="inlineStr"/>
+      <c r="AY51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="AZ51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BB51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BD51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE51" t="inlineStr"/>
+      <c r="BF51" t="inlineStr"/>
+      <c r="BG51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BH51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BJ51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BL51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BN51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ51" t="inlineStr">
+        <is>
+          <t>Attempt 1: [TWS-PEB-002] Collected via tier-1: brand-page (https://www.pebblecart.com/products/striker-buds-tws)</t>
+        </is>
+      </c>
+      <c r="BR51" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>TWS-PEB-003</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Wave Buds</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Wave Buds</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>True wireless stereo earbuds designed for daily audio playback.</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>20 Hours Playtime</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>10mm Drivers</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Type-C Charging</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>125g</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>20 Hours Playtime for extended daily audio listening.</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>10mm Drivers deliver clear sound output for music.</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>125g lightweight design for comfortable daily wear.</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Type-C Charging port for convenient power replenishment.</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-wave-buds)</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/1_1fbe5780-c763-48f9-8221-7ce4daf15c85.jpg?v=1719579309&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr"/>
+      <c r="AF52" t="inlineStr"/>
+      <c r="AG52" t="inlineStr"/>
+      <c r="AH52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr"/>
+      <c r="AJ52" t="inlineStr"/>
+      <c r="AK52" t="inlineStr"/>
+      <c r="AL52" t="inlineStr"/>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>Ready_For_Review</t>
+        </is>
+      </c>
+      <c r="AN52" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AO52" t="inlineStr">
+        <is>
+          <t>Wave</t>
+        </is>
+      </c>
+      <c r="AP52" t="n">
+        <v>2499</v>
+      </c>
+      <c r="AQ52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="AR52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="AT52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU52" t="inlineStr"/>
+      <c r="AV52" t="inlineStr"/>
+      <c r="AW52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="AX52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="AZ52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BB52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BD52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE52" t="inlineStr"/>
+      <c r="BF52" t="inlineStr"/>
+      <c r="BG52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BH52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BJ52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BL52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BN52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ52" t="inlineStr">
+        <is>
+          <t>Attempt 1: [TWS-PEB-003] Collected via tier-1: brand-page (https://www.pebblecart.com/products/pebble-wave-buds)</t>
+        </is>
+      </c>
+      <c r="BR52" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS52" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(tests): add offline regression harness and reset catalogue to powerbanks only
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS52"/>
+  <dimension ref="A1:BS49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10422,639 +10422,6 @@
       </c>
       <c r="BS49" t="inlineStr"/>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>TWS-PEB-001</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>TWS</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Pebble</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Open Loop</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/open-loop</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>Open Loop TWS</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Equipped with environmental noise cancellation for clear audio performance.</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>Environmental Noise Cancellation</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>Features advanced environmental noise cancellation.</t>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>Designed for reliable everyday audio usage.</t>
-        </is>
-      </c>
-      <c r="T50" t="inlineStr"/>
-      <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>tier-1: brand-page (https://www.pebblecart.com/products/open-loop)</t>
-        </is>
-      </c>
-      <c r="W50" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/cdn/shop/files/0_4af773c0-f1d6-4aa9-8aee-9095c75da084.jpg?v=1779955140&amp;width=2048</t>
-        </is>
-      </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y50" t="inlineStr"/>
-      <c r="Z50" t="inlineStr"/>
-      <c r="AA50" t="inlineStr"/>
-      <c r="AB50" t="inlineStr"/>
-      <c r="AC50" t="inlineStr"/>
-      <c r="AD50" t="inlineStr"/>
-      <c r="AE50" t="inlineStr"/>
-      <c r="AF50" t="inlineStr"/>
-      <c r="AG50" t="inlineStr"/>
-      <c r="AH50" t="inlineStr"/>
-      <c r="AI50" t="inlineStr"/>
-      <c r="AJ50" t="inlineStr"/>
-      <c r="AK50" t="inlineStr"/>
-      <c r="AL50" t="inlineStr"/>
-      <c r="AM50" t="inlineStr">
-        <is>
-          <t>Ready_For_Review</t>
-        </is>
-      </c>
-      <c r="AN50" t="inlineStr">
-        <is>
-          <t>local-verified</t>
-        </is>
-      </c>
-      <c r="AO50" t="inlineStr">
-        <is>
-          <t>Open Loop</t>
-        </is>
-      </c>
-      <c r="AP50" t="n">
-        <v>4999</v>
-      </c>
-      <c r="AQ50" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/open-loop</t>
-        </is>
-      </c>
-      <c r="AR50" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS50" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/open-loop</t>
-        </is>
-      </c>
-      <c r="AT50" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU50" t="inlineStr"/>
-      <c r="AV50" t="inlineStr"/>
-      <c r="AW50" t="inlineStr"/>
-      <c r="AX50" t="inlineStr"/>
-      <c r="AY50" t="inlineStr"/>
-      <c r="AZ50" t="inlineStr"/>
-      <c r="BA50" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/open-loop</t>
-        </is>
-      </c>
-      <c r="BB50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC50" t="inlineStr"/>
-      <c r="BD50" t="inlineStr"/>
-      <c r="BE50" t="inlineStr"/>
-      <c r="BF50" t="inlineStr"/>
-      <c r="BG50" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/open-loop</t>
-        </is>
-      </c>
-      <c r="BH50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI50" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/open-loop</t>
-        </is>
-      </c>
-      <c r="BJ50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK50" t="inlineStr"/>
-      <c r="BL50" t="inlineStr"/>
-      <c r="BM50" t="inlineStr"/>
-      <c r="BN50" t="inlineStr"/>
-      <c r="BO50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ50" t="inlineStr">
-        <is>
-          <t>Attempt 1: [TWS-PEB-001] Collected via tier-1: brand-page (https://www.pebblecart.com/products/open-loop)</t>
-        </is>
-      </c>
-      <c r="BR50" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="BS50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>TWS-PEB-002</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>TWS</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Pebble</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>STRIKER Buds</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>STRIKER Buds</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Equipped with advanced bluetooth connectivity and quad mic environmental noise.</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>13mm Drivers</t>
-        </is>
-      </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>Quad Mic ENC</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>Bluetooth v5.4</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>13mm drivers deliver high quality audio output.</t>
-        </is>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>Bluetooth v5.4 provides stable wireless connection.</t>
-        </is>
-      </c>
-      <c r="T51" t="inlineStr">
-        <is>
-          <t>Quad mic ENC ensures clear call performance.</t>
-        </is>
-      </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>Type-C charging port enables fast power replenishment.</t>
-        </is>
-      </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>tier-1: brand-page (https://www.pebblecart.com/products/striker-buds-tws)</t>
-        </is>
-      </c>
-      <c r="W51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/cdn/shop/files/0_e60ef5ad-0831-4ed7-ab69-28c47ef8c9fc.jpg?v=1759139099&amp;width=2048</t>
-        </is>
-      </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y51" t="inlineStr"/>
-      <c r="Z51" t="inlineStr"/>
-      <c r="AA51" t="inlineStr"/>
-      <c r="AB51" t="inlineStr"/>
-      <c r="AC51" t="inlineStr"/>
-      <c r="AD51" t="inlineStr"/>
-      <c r="AE51" t="inlineStr"/>
-      <c r="AF51" t="inlineStr"/>
-      <c r="AG51" t="inlineStr"/>
-      <c r="AH51" t="inlineStr"/>
-      <c r="AI51" t="inlineStr"/>
-      <c r="AJ51" t="inlineStr"/>
-      <c r="AK51" t="inlineStr"/>
-      <c r="AL51" t="inlineStr"/>
-      <c r="AM51" t="inlineStr">
-        <is>
-          <t>Ready_For_Review</t>
-        </is>
-      </c>
-      <c r="AN51" t="inlineStr">
-        <is>
-          <t>local-verified</t>
-        </is>
-      </c>
-      <c r="AO51" t="inlineStr">
-        <is>
-          <t>STRIKER</t>
-        </is>
-      </c>
-      <c r="AP51" t="n">
-        <v>3499</v>
-      </c>
-      <c r="AQ51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="AR51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="AT51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU51" t="inlineStr"/>
-      <c r="AV51" t="inlineStr"/>
-      <c r="AW51" t="inlineStr"/>
-      <c r="AX51" t="inlineStr"/>
-      <c r="AY51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="AZ51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BA51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="BB51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="BD51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE51" t="inlineStr"/>
-      <c r="BF51" t="inlineStr"/>
-      <c r="BG51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="BH51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="BJ51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="BL51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM51" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
-        </is>
-      </c>
-      <c r="BN51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BO51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ51" t="inlineStr">
-        <is>
-          <t>Attempt 1: [TWS-PEB-002] Collected via tier-1: brand-page (https://www.pebblecart.com/products/striker-buds-tws)</t>
-        </is>
-      </c>
-      <c r="BR51" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="BS51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>TWS-PEB-003</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>TWS</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Pebble</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Wave Buds</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>Wave Buds</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>True wireless stereo earbuds designed for daily audio playback.</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>20 Hours Playtime</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>10mm Drivers</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>Type-C Charging</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>125g</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>20 Hours Playtime for extended daily audio listening.</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t>10mm Drivers deliver clear sound output for music.</t>
-        </is>
-      </c>
-      <c r="T52" t="inlineStr">
-        <is>
-          <t>125g lightweight design for comfortable daily wear.</t>
-        </is>
-      </c>
-      <c r="U52" t="inlineStr">
-        <is>
-          <t>Type-C Charging port for convenient power replenishment.</t>
-        </is>
-      </c>
-      <c r="V52" t="inlineStr">
-        <is>
-          <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-wave-buds)</t>
-        </is>
-      </c>
-      <c r="W52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/cdn/shop/files/1_1fbe5780-c763-48f9-8221-7ce4daf15c85.jpg?v=1719579309&amp;width=2048</t>
-        </is>
-      </c>
-      <c r="X52" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="Y52" t="inlineStr"/>
-      <c r="Z52" t="inlineStr"/>
-      <c r="AA52" t="inlineStr"/>
-      <c r="AB52" t="inlineStr"/>
-      <c r="AC52" t="inlineStr"/>
-      <c r="AD52" t="inlineStr"/>
-      <c r="AE52" t="inlineStr"/>
-      <c r="AF52" t="inlineStr"/>
-      <c r="AG52" t="inlineStr"/>
-      <c r="AH52" t="inlineStr"/>
-      <c r="AI52" t="inlineStr"/>
-      <c r="AJ52" t="inlineStr"/>
-      <c r="AK52" t="inlineStr"/>
-      <c r="AL52" t="inlineStr"/>
-      <c r="AM52" t="inlineStr">
-        <is>
-          <t>Ready_For_Review</t>
-        </is>
-      </c>
-      <c r="AN52" t="inlineStr">
-        <is>
-          <t>local-verified</t>
-        </is>
-      </c>
-      <c r="AO52" t="inlineStr">
-        <is>
-          <t>Wave</t>
-        </is>
-      </c>
-      <c r="AP52" t="n">
-        <v>2499</v>
-      </c>
-      <c r="AQ52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="AR52" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="AT52" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU52" t="inlineStr"/>
-      <c r="AV52" t="inlineStr"/>
-      <c r="AW52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="AX52" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="AZ52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BA52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="BB52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BC52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="BD52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BE52" t="inlineStr"/>
-      <c r="BF52" t="inlineStr"/>
-      <c r="BG52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="BH52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="BJ52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BK52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="BL52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM52" t="inlineStr">
-        <is>
-          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
-        </is>
-      </c>
-      <c r="BN52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BO52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP52" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ52" t="inlineStr">
-        <is>
-          <t>Attempt 1: [TWS-PEB-003] Collected via tier-1: brand-page (https://www.pebblecart.com/products/pebble-wave-buds)</t>
-        </is>
-      </c>
-      <c r="BR52" t="inlineStr">
-        <is>
-          <t>gemini</t>
-        </is>
-      </c>
-      <c r="BS52" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(jbl): purge JBL test rows, run reports, and brand configuration for clean test
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS49"/>
+  <dimension ref="A1:BS52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10422,6 +10422,487 @@
       </c>
       <c r="BS49" t="inlineStr"/>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TWS-PEB-001</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Openloop</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr"/>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr"/>
+      <c r="AI50" t="inlineStr"/>
+      <c r="AJ50" t="inlineStr"/>
+      <c r="AK50" t="inlineStr"/>
+      <c r="AL50" t="inlineStr">
+        <is>
+          <t>Skipped: Skipped: All spec tiers exhausted (including Vision) without finding technical specifications</t>
+        </is>
+      </c>
+      <c r="AM50" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="AN50" t="inlineStr"/>
+      <c r="AO50" t="inlineStr">
+        <is>
+          <t>Openloop</t>
+        </is>
+      </c>
+      <c r="AP50" t="n">
+        <v>4999</v>
+      </c>
+      <c r="AQ50" t="inlineStr"/>
+      <c r="AR50" t="inlineStr"/>
+      <c r="AS50" t="inlineStr"/>
+      <c r="AT50" t="inlineStr"/>
+      <c r="AU50" t="inlineStr"/>
+      <c r="AV50" t="inlineStr"/>
+      <c r="AW50" t="inlineStr"/>
+      <c r="AX50" t="inlineStr"/>
+      <c r="AY50" t="inlineStr"/>
+      <c r="AZ50" t="inlineStr"/>
+      <c r="BA50" t="inlineStr"/>
+      <c r="BB50" t="inlineStr"/>
+      <c r="BC50" t="inlineStr"/>
+      <c r="BD50" t="inlineStr"/>
+      <c r="BE50" t="inlineStr"/>
+      <c r="BF50" t="inlineStr"/>
+      <c r="BG50" t="inlineStr"/>
+      <c r="BH50" t="inlineStr"/>
+      <c r="BI50" t="inlineStr"/>
+      <c r="BJ50" t="inlineStr"/>
+      <c r="BK50" t="inlineStr"/>
+      <c r="BL50" t="inlineStr"/>
+      <c r="BM50" t="inlineStr"/>
+      <c r="BN50" t="inlineStr"/>
+      <c r="BO50" t="inlineStr"/>
+      <c r="BP50" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ50" t="inlineStr">
+        <is>
+          <t>Attempt 1: [TWS-PEB-001] SKIPPED: All tiers exhausted</t>
+        </is>
+      </c>
+      <c r="BR50" t="inlineStr"/>
+      <c r="BS50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TWS-PEB-002</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>STRIKER Buds</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>STRIKER Buds</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Compact wireless audio device equipped with Type-C connectivity.</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Type-C</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Type-C port included for universal charging access.</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>True wireless stereo design for portable listening.</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/striker-buds-tws)</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/0_e60ef5ad-0831-4ed7-ab69-28c47ef8c9fc.jpg?v=1759139099&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr"/>
+      <c r="AF51" t="inlineStr"/>
+      <c r="AG51" t="inlineStr"/>
+      <c r="AH51" t="inlineStr"/>
+      <c r="AI51" t="inlineStr"/>
+      <c r="AJ51" t="inlineStr"/>
+      <c r="AK51" t="inlineStr"/>
+      <c r="AL51" t="inlineStr"/>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AN51" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AO51" t="inlineStr">
+        <is>
+          <t>STRIKER</t>
+        </is>
+      </c>
+      <c r="AP51" t="n">
+        <v>3499</v>
+      </c>
+      <c r="AQ51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="AR51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="AT51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU51" t="inlineStr"/>
+      <c r="AV51" t="inlineStr"/>
+      <c r="AW51" t="inlineStr"/>
+      <c r="AX51" t="inlineStr"/>
+      <c r="AY51" t="inlineStr"/>
+      <c r="AZ51" t="inlineStr"/>
+      <c r="BA51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BB51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC51" t="inlineStr"/>
+      <c r="BD51" t="inlineStr"/>
+      <c r="BE51" t="inlineStr"/>
+      <c r="BF51" t="inlineStr"/>
+      <c r="BG51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BH51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI51" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/striker-buds-tws</t>
+        </is>
+      </c>
+      <c r="BJ51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK51" t="inlineStr"/>
+      <c r="BL51" t="inlineStr"/>
+      <c r="BM51" t="inlineStr"/>
+      <c r="BN51" t="inlineStr"/>
+      <c r="BO51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ51" t="inlineStr">
+        <is>
+          <t>Attempt 1: [TWS-PEB-002] Collected via tier-1: brand-page (https://www.pebblecart.com/products/striker-buds-tws)</t>
+        </is>
+      </c>
+      <c r="BR51" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>TWS-PEB-003</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Pebble</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Wave Buds</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Wave Buds</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>True wireless stereo audio device with Type-C connectivity.</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Type-C</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>125g</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>125g total weight designed for comfortable everyday use.</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Type-C charging port included for modern power delivery.</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://www.pebblecart.com/products/pebble-wave-buds)</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/cdn/shop/files/1_1fbe5780-c763-48f9-8221-7ce4daf15c85.jpg?v=1719579309&amp;width=2048</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr"/>
+      <c r="AF52" t="inlineStr"/>
+      <c r="AG52" t="inlineStr"/>
+      <c r="AH52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr"/>
+      <c r="AJ52" t="inlineStr"/>
+      <c r="AK52" t="inlineStr"/>
+      <c r="AL52" t="inlineStr"/>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AN52" t="inlineStr">
+        <is>
+          <t>brand-product-page</t>
+        </is>
+      </c>
+      <c r="AO52" t="inlineStr">
+        <is>
+          <t>Wave</t>
+        </is>
+      </c>
+      <c r="AP52" t="n">
+        <v>2499</v>
+      </c>
+      <c r="AQ52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="AR52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="AT52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU52" t="inlineStr"/>
+      <c r="AV52" t="inlineStr"/>
+      <c r="AW52" t="inlineStr"/>
+      <c r="AX52" t="inlineStr"/>
+      <c r="AY52" t="inlineStr"/>
+      <c r="AZ52" t="inlineStr"/>
+      <c r="BA52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BB52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BD52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE52" t="inlineStr"/>
+      <c r="BF52" t="inlineStr"/>
+      <c r="BG52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BH52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI52" t="inlineStr">
+        <is>
+          <t>https://www.pebblecart.com/products/pebble-wave-buds</t>
+        </is>
+      </c>
+      <c r="BJ52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK52" t="inlineStr"/>
+      <c r="BL52" t="inlineStr"/>
+      <c r="BM52" t="inlineStr"/>
+      <c r="BN52" t="inlineStr"/>
+      <c r="BO52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ52" t="inlineStr">
+        <is>
+          <t>Attempt 1: [TWS-PEB-003] Collected via tier-1: brand-page (https://www.pebblecart.com/products/pebble-wave-buds)</t>
+        </is>
+      </c>
+      <c r="BR52" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS52" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(jbl): clean up JBL test rows and brand configuration for fresh frontend testing
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -4278,18 +4278,18 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Portronics Luxcell B12</t>
+          <t>Luxcell B12</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Compact power bank equipped with multiple device charging ports.</t>
+          <t>Compact power delivery solution for daily mobile charging needs.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
-          <t>10000 mAh</t>
+          <t>10000mAh</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -4306,17 +4306,17 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>10000 mAh capacity stores backup power for devices.</t>
+          <t>10000mAh capacity supports multiple full device charges.</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>12W Fast Charging delivers quick power output.</t>
+          <t>12W fast charging delivers rapid power replenishment.</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Type-C input allows standard cable connection.</t>
+          <t>Type-C and USB-A dual ports connect multiple devices.</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
@@ -4348,11 +4348,7 @@
       <c r="AI21" t="inlineStr"/>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr"/>
-      <c r="AL21" t="inlineStr">
-        <is>
-          <t>Partial specifications: 1 of 5 specs empty (weight)</t>
-        </is>
-      </c>
+      <c r="AL21" t="inlineStr"/>
       <c r="AM21" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4360,7 +4356,7 @@
       </c>
       <c r="AN21" t="inlineStr">
         <is>
-          <t>brand-product-page</t>
+          <t>local-verified</t>
         </is>
       </c>
       <c r="AO21" t="inlineStr">
@@ -5425,6 +5421,7 @@
 Cleaned Display_Name to 'nan'
 Attempt 1: [PB-POR-008] SKIPPED: All tiers exhausted
 Cleaned Display_Name to 'nan'
+Cleaned Display_Name to 'nan'
 Cleaned Display_Name to 'nan'</t>
         </is>
       </c>
@@ -5978,6 +5975,7 @@
         <is>
           <t>Attempt 1: [PB-POR-011] Collected via tier-1: brand-page (https://www.portronics.com/products/power-shutter)
 Attempt 1: No automated fix available for flags: ['Duplicate image asset: identical file hash to product [PB-POR-004]']
+Cleaned Display_Name to 'nan'
 Cleaned Display_Name to 'nan'
 Cleaned Display_Name to 'nan'
 Cleaned Display_Name to 'nan'</t>
@@ -6092,6 +6090,7 @@
       <c r="BQ30" t="inlineStr">
         <is>
           <t>Attempt 1: [PB-POR-012] BLOCKED: All tiers exhausted
+Cleaned Display_Name to 'nan'
 Cleaned Display_Name to 'nan'
 Cleaned Display_Name to 'nan'
 Cleaned Display_Name to 'nan'</t>

</xml_diff>

<commit_message>
feat(catalogue): update brand defaults and catalogue data with JBL TWS
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS52"/>
+  <dimension ref="A1:BS55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10902,6 +10902,606 @@
       </c>
       <c r="BS52" t="inlineStr"/>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TWS-JBL-001</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>JBL</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Tune Beam 2</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Tune Beam 2</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Audio products designed for party time and study time.</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Bluetooth audio products designed for study and party time.</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Designed for party time, study time, and anytime listening.</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://in.jbl.com)</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>needs-better-image</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr"/>
+      <c r="Z53" t="inlineStr"/>
+      <c r="AA53" t="inlineStr"/>
+      <c r="AB53" t="inlineStr"/>
+      <c r="AC53" t="inlineStr"/>
+      <c r="AD53" t="inlineStr"/>
+      <c r="AE53" t="inlineStr"/>
+      <c r="AF53" t="inlineStr"/>
+      <c r="AG53" t="inlineStr"/>
+      <c r="AH53" t="inlineStr"/>
+      <c r="AI53" t="inlineStr"/>
+      <c r="AJ53" t="inlineStr"/>
+      <c r="AK53" t="inlineStr"/>
+      <c r="AL53" t="inlineStr">
+        <is>
+          <t>Specifications derived directly from verified product description</t>
+        </is>
+      </c>
+      <c r="AM53" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AN53" t="inlineStr">
+        <is>
+          <t>amazon.in/dp/B0CHVTF8M7 (Score 2/10: Wrong brand detected: 'Unknown' (expected 'JBL'))</t>
+        </is>
+      </c>
+      <c r="AO53" t="inlineStr">
+        <is>
+          <t>Tune Beam</t>
+        </is>
+      </c>
+      <c r="AP53" t="n">
+        <v>11999</v>
+      </c>
+      <c r="AQ53" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com</t>
+        </is>
+      </c>
+      <c r="AR53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS53" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com</t>
+        </is>
+      </c>
+      <c r="AT53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU53" t="inlineStr"/>
+      <c r="AV53" t="inlineStr"/>
+      <c r="AW53" t="inlineStr"/>
+      <c r="AX53" t="inlineStr"/>
+      <c r="AY53" t="inlineStr"/>
+      <c r="AZ53" t="inlineStr"/>
+      <c r="BA53" t="inlineStr"/>
+      <c r="BB53" t="inlineStr"/>
+      <c r="BC53" t="inlineStr"/>
+      <c r="BD53" t="inlineStr"/>
+      <c r="BE53" t="inlineStr"/>
+      <c r="BF53" t="inlineStr"/>
+      <c r="BG53" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com</t>
+        </is>
+      </c>
+      <c r="BH53" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI53" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com</t>
+        </is>
+      </c>
+      <c r="BJ53" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK53" t="inlineStr"/>
+      <c r="BL53" t="inlineStr"/>
+      <c r="BM53" t="inlineStr"/>
+      <c r="BN53" t="inlineStr"/>
+      <c r="BO53" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP53" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ53" t="inlineStr">
+        <is>
+          <t>Attempt 1: [TWS-JBL-001] Collected via tier-1: brand-page (https://in.jbl.com)</t>
+        </is>
+      </c>
+      <c r="BR53" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TWS-JBL-002</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>JBL</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Tour Pro 3</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Tour Pro 3</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>True wireless earbuds with smart charging case and spatial audio.</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>44 Hours Playtime</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>10.2mm Drivers</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Active Noise Cancellation</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Bluetooth v5.3</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>10.2mm Drivers deliver legendary hybrid dual-driver sound.</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>44 Hours Playtime provides extended everyday listening.</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Bluetooth v5.3 connects with any compatible device.</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Active Noise Cancellation tunes out the surrounding world.</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://in.jbl.com/TOUR-PRO-3.html)</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr"/>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr"/>
+      <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr"/>
+      <c r="AD54" t="inlineStr"/>
+      <c r="AE54" t="inlineStr"/>
+      <c r="AF54" t="inlineStr"/>
+      <c r="AG54" t="inlineStr"/>
+      <c r="AH54" t="inlineStr"/>
+      <c r="AI54" t="inlineStr"/>
+      <c r="AJ54" t="inlineStr"/>
+      <c r="AK54" t="inlineStr"/>
+      <c r="AL54" t="inlineStr"/>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AN54" t="inlineStr">
+        <is>
+          <t>local-verified</t>
+        </is>
+      </c>
+      <c r="AO54" t="inlineStr">
+        <is>
+          <t>Tour</t>
+        </is>
+      </c>
+      <c r="AP54" t="n">
+        <v>29999</v>
+      </c>
+      <c r="AQ54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="AR54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="AT54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU54" t="inlineStr"/>
+      <c r="AV54" t="inlineStr"/>
+      <c r="AW54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="AX54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="AZ54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="BB54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="BD54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE54" t="inlineStr"/>
+      <c r="BF54" t="inlineStr"/>
+      <c r="BG54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="BH54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="BJ54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="BL54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM54" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/TOUR-PRO-3.html</t>
+        </is>
+      </c>
+      <c r="BN54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP54" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ54" t="inlineStr">
+        <is>
+          <t>Collected via tier-1: brand-page (https://in.jbl.com/TOUR-PRO-3.html)
+[Review Re-run 1]: Re-collected due to review critique: The specs are completely scrambled: 'output' lists driver size, 'ports' lists a feature (Active Noise Cancellation), and 'weight' lists a connectivity protocol (Bluetooth v5.3)., Copy mismatch: The copy correctly describes the JBL Tour Pro 3 earbuds, but the extracted technical specs are misaligned and mapping incorrect data categories (e.g. putting bluetooth version under weight).</t>
+        </is>
+      </c>
+      <c r="BR54" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>TWS-JBL-003</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>TWS</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>JBL</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Live Beam 3</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/LIVEBEAM3.html</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Live Beam 3</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>True wireless earbuds featuring adaptive noise cancelling and smart case.</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>48 Hours Playtime</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>10mm Drivers</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Active Noise Cancellation</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>48 hours total playback plus wireless charging.</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>6 mics for calls you can customize yourself.</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>tier-1: brand-page (https://in.jbl.com/LIVEBEAM3.html)</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr"/>
+      <c r="Z55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr"/>
+      <c r="AD55" t="inlineStr"/>
+      <c r="AE55" t="inlineStr"/>
+      <c r="AF55" t="inlineStr"/>
+      <c r="AG55" t="inlineStr"/>
+      <c r="AH55" t="inlineStr"/>
+      <c r="AI55" t="inlineStr"/>
+      <c r="AJ55" t="inlineStr"/>
+      <c r="AK55" t="inlineStr"/>
+      <c r="AL55" t="inlineStr">
+        <is>
+          <t>Image sourced from secondary channel: amazon.in/dp/B0GSCDC3LT</t>
+        </is>
+      </c>
+      <c r="AM55" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="AN55" t="inlineStr">
+        <is>
+          <t>amazon.in/dp/B0GSCDC3LT</t>
+        </is>
+      </c>
+      <c r="AO55" t="inlineStr">
+        <is>
+          <t>Live Beam</t>
+        </is>
+      </c>
+      <c r="AP55" t="n">
+        <v>24999</v>
+      </c>
+      <c r="AQ55" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/LIVEBEAM3.html</t>
+        </is>
+      </c>
+      <c r="AR55" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS55" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/LIVEBEAM3.html</t>
+        </is>
+      </c>
+      <c r="AT55" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU55" t="inlineStr"/>
+      <c r="AV55" t="inlineStr"/>
+      <c r="AW55" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/LIVEBEAM3.html</t>
+        </is>
+      </c>
+      <c r="AX55" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY55" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/LIVEBEAM3.html</t>
+        </is>
+      </c>
+      <c r="AZ55" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA55" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/LIVEBEAM3.html</t>
+        </is>
+      </c>
+      <c r="BB55" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC55" t="inlineStr"/>
+      <c r="BD55" t="inlineStr"/>
+      <c r="BE55" t="inlineStr"/>
+      <c r="BF55" t="inlineStr"/>
+      <c r="BG55" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/LIVEBEAM3.html</t>
+        </is>
+      </c>
+      <c r="BH55" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI55" t="inlineStr">
+        <is>
+          <t>https://in.jbl.com/LIVEBEAM3.html</t>
+        </is>
+      </c>
+      <c r="BJ55" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK55" t="inlineStr"/>
+      <c r="BL55" t="inlineStr"/>
+      <c r="BM55" t="inlineStr"/>
+      <c r="BN55" t="inlineStr"/>
+      <c r="BO55" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP55" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ55" t="inlineStr">
+        <is>
+          <t>Attempt 1: [TWS-JBL-003] Collected via tier-1: brand-page (https://in.jbl.com/LIVEBEAM3.html)</t>
+        </is>
+      </c>
+      <c r="BR55" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="BS55" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(jbl): re-collect verified brand images for JBL Tour Pro 3 and Tune Beam 2
</commit_message>
<xml_diff>
--- a/data/catalogue_data.xlsx
+++ b/data/catalogue_data.xlsx
@@ -10968,7 +10968,7 @@
       <c r="W53" t="inlineStr"/>
       <c r="X53" t="inlineStr">
         <is>
-          <t>needs-better-image</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="Y53" t="inlineStr"/>
@@ -10996,7 +10996,7 @@
       </c>
       <c r="AN53" t="inlineStr">
         <is>
-          <t>amazon.in/dp/B0CHVTF8M7 (Score 2/10: Wrong brand detected: 'Unknown' (expected 'JBL'))</t>
+          <t>amazon.in/dp/B0DK3W2XK3</t>
         </is>
       </c>
       <c r="AO53" t="inlineStr">
@@ -11059,7 +11059,7 @@
         <v>3</v>
       </c>
       <c r="BP53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BQ53" t="inlineStr">
         <is>
@@ -11187,7 +11187,7 @@
       </c>
       <c r="AN54" t="inlineStr">
         <is>
-          <t>local-verified</t>
+          <t>amazon.in/dp/B0D44H2RG3</t>
         </is>
       </c>
       <c r="AO54" t="inlineStr">
@@ -11283,10 +11283,10 @@
         <v>1</v>
       </c>
       <c r="BO54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BP54" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BQ54" t="inlineStr">
         <is>

</xml_diff>